<commit_message>
refactor: standardize Excel headers to Activity Description and CR-DM-PDM ID across backend logic and API responses.
</commit_message>
<xml_diff>
--- a/redmine-logger/backend/user_data/lumiqshubh23/git_commits.xlsx
+++ b/redmine-logger/backend/user_data/lumiqshubh23/git_commits.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,7 +407,7 @@
         <v>Commit</v>
       </c>
       <c r="C1" t="str">
-        <v>AI Task</v>
+        <v>Activity Description</v>
       </c>
       <c r="D1" t="str">
         <v>Type</v>
@@ -420,6 +420,9 @@
       </c>
       <c r="G1" t="str">
         <v>Branch</v>
+      </c>
+      <c r="H1" t="str">
+        <v>AI Task</v>
       </c>
     </row>
     <row r="2">
@@ -427,22 +430,22 @@
         <v>2026-03-31</v>
       </c>
       <c r="B2" t="str">
-        <v>dynamic heading added for nomiee</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Dynamic Heading Implementation for Nominee</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="D2" t="str">
-        <v>Feature</v>
+        <v>Meeting</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F2" t="str">
-        <v>d3ea10c7a2788c713a29f895502e35ae8edd3868</v>
+        <v>N/A</v>
       </c>
       <c r="G2" t="str">
-        <v>smartGuaranteedPension-frontend</v>
+        <v>N/A</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="3">
@@ -450,401 +453,401 @@
         <v>2026-03-31</v>
       </c>
       <c r="B3" t="str">
-        <v>annur hide</v>
+        <v>Merge branch 'CR-36689-cpf' into secureInvestPlan-frontend</v>
       </c>
       <c r="C3" t="str">
         <v>Enhance Video Verification UI</v>
       </c>
       <c r="D3" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F3" t="str">
-        <v>9f4b41ecdd9cd9d1c7b5100c0502cb80b744e607</v>
+        <v>2a45016e7d08ac1ff1deebddea70d31615dac6ce</v>
       </c>
       <c r="G3" t="str">
-        <v>youngTermPlan-frontend</v>
+        <v>secureInvestPlan-frontend</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04-02</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B4" t="str">
-        <v>SGP dynamic heading restore</v>
+        <v>Merge branch 'CR-36689-ytp' into youngTermPlan-frontend</v>
       </c>
       <c r="C4" t="str">
-        <v>Enhance Dynamic Heading Logic</v>
+        <v>Integrate Video Verification Update</v>
       </c>
       <c r="D4" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F4" t="str">
-        <v>b537a3e12f502977f59688c70e1beea90d2fec35</v>
+        <v>a578e730156cffe058e79f7ebf3bd8ab2f5a7224</v>
       </c>
       <c r="G4" t="str">
-        <v>smartGuaranteedPension-frontend</v>
+        <v>secureInvestPlan-frontend</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04-03</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B5" t="str">
-        <v>upload proceed now bg color fix</v>
+        <v>Merge branch 'smartGuaranteedPension-frontend' of https://github.com/lumiqai/ISNP into smartGuaranteedPension-frontend</v>
       </c>
       <c r="C5" t="str">
-        <v>Fix Background Color for Disabled Button</v>
+        <v>Integrate Frontend Changes from Smart Guaranteed Pension</v>
       </c>
       <c r="D5" t="str">
-        <v>Bug Fix</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>0.27</v>
       </c>
       <c r="F5" t="str">
-        <v>07ce50fc8b2eee8ef8b950d4fca44b76d5d2f0e8</v>
+        <v>0fd712bf8b1347c3fe22c1895d159849224e4b53</v>
       </c>
       <c r="G5" t="str">
-        <v>secureInvestPlan-frontend</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04-03</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B6" t="str">
-        <v>upload proceed now bg color fix</v>
+        <v>Merge branch 'CR-36689-sgp' into smartGuaranteedPension-frontend</v>
       </c>
       <c r="C6" t="str">
-        <v>Fix Background Color for Disabled Button</v>
+        <v>Integrate Smart Guaranteed Pension Features</v>
       </c>
       <c r="D6" t="str">
-        <v>Bug Fix</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="F6" t="str">
-        <v>46a28661cc5dac4485d580118e4e833aedd9e43d</v>
+        <v>063e7e3b5addac7da001066ff1300f3b0afb9570</v>
       </c>
       <c r="G6" t="str">
-        <v>3-april-release-secureInvest-2026</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04-03</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B7" t="str">
-        <v>for EQUITAS no setIsLaMinor check</v>
+        <v>Merge branch 'CR-36689-sgp' of https://github.com/lumiqai/ISNP into CR-36689-sgp</v>
       </c>
       <c r="C7" t="str">
-        <v>Update Age Check for EQUITAS Channel</v>
+        <v>Integrate Account Holder Metadata Fields</v>
       </c>
       <c r="D7" t="str">
-        <v>Bug Fix</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F7" t="str">
-        <v>00769029756bf4bd56ff6a427ae499eeae16b960</v>
+        <v>4b7b4044c099e3c8ac8cc250deb59dfb935a53be</v>
       </c>
       <c r="G7" t="str">
-        <v>3-april-release-p4f-2026</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04-08</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B8" t="str">
-        <v>penny drop api integration</v>
+        <v>dynamic heading added for nomiee</v>
       </c>
       <c r="C8" t="str">
-        <v>Integrate Penny Drop API for Nominees</v>
+        <v>Dynamic Party Labels for Headings</v>
       </c>
       <c r="D8" t="str">
         <v>Feature</v>
       </c>
       <c r="E8">
-        <v>8</v>
+        <v>0.53</v>
       </c>
       <c r="F8" t="str">
-        <v>02a0346b85c21edd1a9d014673cfe4de5b62319a</v>
+        <v>d3ea10c7a2788c713a29f895502e35ae8edd3868</v>
       </c>
       <c r="G8" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04-14</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B9" t="str">
-        <v>ComponentCmpTagToggleSwitch fix</v>
+        <v>Merge branch 'CR-36689-sgp' into smartGuaranteedPension-frontend</v>
       </c>
       <c r="C9" t="str">
-        <v>Fix Address Type Default Values</v>
+        <v>Integrate Video Verification Completion Indicator</v>
       </c>
       <c r="D9" t="str">
-        <v>Bug Fix</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F9" t="str">
-        <v>2b27bcb1a3dbf6ee69378b7ac249cfead456cb64</v>
+        <v>f315e23defbbd7f4cc07a3baa33ccc8ed06078e0</v>
       </c>
       <c r="G9" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04-14</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B10" t="str">
-        <v>staff discount key fix</v>
+        <v>Merge branch 'CR-36689-ytp' into youngTermPlan-frontend</v>
       </c>
       <c r="C10" t="str">
-        <v>Staff Discount Key Configuration Update</v>
+        <v>Integrate Video Verification Feedback</v>
       </c>
       <c r="D10" t="str">
-        <v>Bug Fix</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F10" t="str">
-        <v>dc031ec605640971539a9bc93b4c0f976637469d</v>
+        <v>5d58648336b919def5889797564c1faf36414ead</v>
       </c>
       <c r="G10" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04-14</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B11" t="str">
-        <v>changemedicalquestionvalue</v>
+        <v>Merge branch 'CR-36689-cpf' into promise4LifePlan-frontend</v>
       </c>
       <c r="C11" t="str">
-        <v>Update Medical Question Response Values</v>
+        <v>Enhance Video Verification Notification</v>
       </c>
       <c r="D11" t="str">
-        <v>Refactor</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F11" t="str">
-        <v>c7392d4b62dbde0eb773ec17867342d36088dff7</v>
+        <v>b32e48c4b1ab200f4a437f2f52eb98c361ad23f4</v>
       </c>
       <c r="G11" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>promise4LifePlan-frontend</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04-17</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B12" t="str">
-        <v>inital structure ready</v>
+        <v>Merge branch 'CR-36689-cpf' into promise4FuturePlan-frontend</v>
       </c>
       <c r="C12" t="str">
-        <v>Implement Initial Product Details Structure</v>
+        <v>Enhance Video Verification UI</v>
       </c>
       <c r="D12" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>0.53</v>
       </c>
       <c r="F12" t="str">
-        <v>f901a74de1fd96ae6f1aef0b8319e4eddb2d5773</v>
+        <v>cf412e12e7b1da80d2d23c0ce52679e410b61ff7</v>
       </c>
       <c r="G12" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>promise4FuturePlan-frontend</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04-20</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B13" t="str">
-        <v>add</v>
+        <v>Merge branch 'CR-36689-cpf' into igfp-frontend</v>
       </c>
       <c r="C13" t="str">
-        <v>Implement Environment Configuration and Payment Gateway Flow</v>
+        <v>Enhance Video Verification UI</v>
       </c>
       <c r="D13" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E13">
-        <v>8</v>
+        <v>0.53</v>
       </c>
       <c r="F13" t="str">
-        <v>375c93478bef64cdb7e9a780bb6d1e68c1109902</v>
+        <v>9a1c362294112557eeedbffe9b4519fcd9b12743</v>
       </c>
       <c r="G13" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>igfp-frontend</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04-20</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B14" t="str">
-        <v>add</v>
+        <v>Merge branch 'CR-36689-cpf' into titaniumPlusPlan-frontend</v>
       </c>
       <c r="C14" t="str">
-        <v>Implement Developer Console Feature</v>
+        <v>Integrate Video Verification Feedback</v>
       </c>
       <c r="D14" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E14">
-        <v>8</v>
+        <v>0.53</v>
       </c>
       <c r="F14" t="str">
-        <v>4d0fd3607c349a8d69f17422ad68d36d3b26ded0</v>
+        <v>81dacea5dcb640aa8adf70f5d874a134e11cc94c</v>
       </c>
       <c r="G14" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>titaniumPlusPlan-frontend</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04-20</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B15" t="str">
-        <v>secureInvest-riderAdded</v>
+        <v>Merge branch 'CR-36689-cpf' into gain-frontend</v>
       </c>
       <c r="C15" t="str">
-        <v>Enhance Secure Invest Rider Options</v>
+        <v>Integrate Video Verification Completion Status</v>
       </c>
       <c r="D15" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>0.53</v>
       </c>
       <c r="F15" t="str">
-        <v>fefbe626c36732b9363c5c98c9df68475c3c8b1e</v>
+        <v>bd1a528cd95f824ab41885ba470f894c5576ef31</v>
       </c>
       <c r="G15" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>gain-frontend</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04-22</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B16" t="str">
-        <v>fix: sync package-lock with package.json</v>
+        <v>Merge branch 'CR-36689-ytp' into youngTermPlan-frontend</v>
       </c>
       <c r="C16" t="str">
-        <v>Synchronize package-lock with package.json</v>
+        <v>Enhance Video Verification UI</v>
       </c>
       <c r="D16" t="str">
-        <v>Bug Fix</v>
+        <v>Feature</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0.53</v>
       </c>
       <c r="F16" t="str">
-        <v>d6dd30dc3c8303c114e9a2e62afbd6a30a3a969d</v>
+        <v>fbed8454db25776abda5d01266e09da8d74a9c42</v>
       </c>
       <c r="G16" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>youngTermPlan-frontend</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04-22</v>
+        <v>2026-03-31</v>
       </c>
       <c r="B17" t="str">
-        <v>package json fix</v>
+        <v>annur hide</v>
       </c>
       <c r="C17" t="str">
-        <v>Package Configuration Correction</v>
+        <v>Enhance Video Verification UI</v>
       </c>
       <c r="D17" t="str">
-        <v>Bug Fix</v>
+        <v>Feature</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>0.57</v>
       </c>
       <c r="F17" t="str">
-        <v>2704e1bc206feb7affebb6a2eb2df8c10ba0ea55</v>
+        <v>9f4b41ecdd9cd9d1c7b5100c0502cb80b744e607</v>
       </c>
       <c r="G17" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>youngTermPlan-frontend</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04-22</v>
+        <v>2026-04-02</v>
       </c>
       <c r="B18" t="str">
-        <v>sync package.json issue</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Address Package.json Synchronization Issue</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="D18" t="str">
-        <v>Bug Fix</v>
+        <v>Meeting</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="str">
-        <v>c05a99adf2c8c7ff431706c387f79cc9e91fc4b4</v>
+        <v>N/A</v>
       </c>
       <c r="G18" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04-22</v>
+        <v>2026-04-02</v>
       </c>
       <c r="B19" t="str">
-        <v>rider premium mapping</v>
+        <v>Merge remote-tracking branch 'origin/CR-36689-sgp' into smartGuaranteedPension-frontend</v>
       </c>
       <c r="C19" t="str">
-        <v>Implement Rider Premium Mapping Utility</v>
+        <v>Integrate Proposer and Annuitant Details</v>
       </c>
       <c r="D19" t="str">
-        <v>Feature</v>
+        <v>Integration/Merge</v>
       </c>
       <c r="E19">
         <v>4</v>
       </c>
       <c r="F19" t="str">
-        <v>303affc8a58d89cd5fa4a833ae47d83064bd0d1f</v>
+        <v>8a0f938e39a892ae41e3712b270821e2ba92f58a</v>
       </c>
       <c r="G19" t="str">
-        <v>insure/secureInvest2.0</v>
+        <v>smartGuaranteedPension-frontend</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04-22</v>
+        <v>2026-04-02</v>
       </c>
       <c r="B20" t="str">
-        <v>BI called with rider</v>
+        <v>SGP dynamic heading restore</v>
       </c>
       <c r="C20" t="str">
-        <v>Enhance Critical Illness Rider Features</v>
+        <v>Dynamic Heading Restoration for Annuitants</v>
       </c>
       <c r="D20" t="str">
         <v>Feature</v>
@@ -853,15 +856,1027 @@
         <v>4</v>
       </c>
       <c r="F20" t="str">
+        <v>b537a3e12f502977f59688c70e1beea90d2fec35</v>
+      </c>
+      <c r="G20" t="str">
+        <v>smartGuaranteedPension-frontend</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-04-03</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G21" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-04-03</v>
+      </c>
+      <c r="B22" t="str">
+        <v>upload proceed now bg color fix</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Improve Button Appearance on Disable</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22" t="str">
+        <v>07ce50fc8b2eee8ef8b950d4fca44b76d5d2f0e8</v>
+      </c>
+      <c r="G22" t="str">
+        <v>secureInvestPlan-frontend</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-04-03</v>
+      </c>
+      <c r="B23" t="str">
+        <v>upload proceed now bg color fix</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Fix Background Color for Disabled Buttons</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+      <c r="F23" t="str">
+        <v>46a28661cc5dac4485d580118e4e833aedd9e43d</v>
+      </c>
+      <c r="G23" t="str">
+        <v>3-april-release-secureInvest-2026</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-04-03</v>
+      </c>
+      <c r="B24" t="str">
+        <v>for EQUITAS no setIsLaMinor check</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Conditional Check for Minor Status</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E24">
+        <v>4</v>
+      </c>
+      <c r="F24" t="str">
+        <v>00769029756bf4bd56ff6a427ae499eeae16b960</v>
+      </c>
+      <c r="G24" t="str">
+        <v>3-april-release-p4f-2026</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-04-06</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G25" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-04-06</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/ISNP into insure/develop</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Merge Branch 'insure/develop'</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E26">
+        <v>8</v>
+      </c>
+      <c r="F26" t="str">
+        <v>d93ae5f941d87ea5732797d2c4cfddaf5866cede</v>
+      </c>
+      <c r="G26" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-04-08</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G27" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-04-08</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Merge branch 'pennydropIntegration' into insure/develop</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Integrate Penny Drop Validation for Nominees</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E28">
+        <v>5.33</v>
+      </c>
+      <c r="F28" t="str">
+        <v>3ceae4cc67801e95eb56db7c177c990c72236619</v>
+      </c>
+      <c r="G28" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-04-08</v>
+      </c>
+      <c r="B29" t="str">
+        <v>penny drop api integration</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Integrate Penny Drop Validation API</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E29">
+        <v>2.67</v>
+      </c>
+      <c r="F29" t="str">
+        <v>02a0346b85c21edd1a9d014673cfe4de5b62319a</v>
+      </c>
+      <c r="G29" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G30" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/ISNP into insure/develop</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Integrate New Risky Hobbies Components</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E31">
+        <v>2.67</v>
+      </c>
+      <c r="F31" t="str">
+        <v>e6ea46bcf8d7df1a21e4c443a0920d77e25033d1</v>
+      </c>
+      <c r="G31" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B32" t="str">
+        <v>ComponentCmpTagToggleSwitch fix</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Update Address Type Default Values</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E32">
+        <v>1.33</v>
+      </c>
+      <c r="F32" t="str">
+        <v>2b27bcb1a3dbf6ee69378b7ac249cfead456cb64</v>
+      </c>
+      <c r="G32" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/ISNP into insure/develop</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Enhance Date Input Component Logic</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E33">
+        <v>1.33</v>
+      </c>
+      <c r="F33" t="str">
+        <v>9bf249b9e60b5e0cf8f1735f41147f49fe6f6fc3</v>
+      </c>
+      <c r="G33" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B34" t="str">
+        <v>staff discount key fix</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Update Staff Discount Key Logic</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Refactor</v>
+      </c>
+      <c r="E34">
+        <v>1.33</v>
+      </c>
+      <c r="F34" t="str">
+        <v>dc031ec605640971539a9bc93b4c0f976637469d</v>
+      </c>
+      <c r="G34" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B35" t="str">
+        <v>changemedicalquestionvalue</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Update Medical Question Value Types</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Refactor</v>
+      </c>
+      <c r="E35">
+        <v>1.34</v>
+      </c>
+      <c r="F35" t="str">
+        <v>c7392d4b62dbde0eb773ec17867342d36088dff7</v>
+      </c>
+      <c r="G35" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G36" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="B37" t="str">
+        <v>inital structure ready</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Initial Structure Setup for Insurance Details</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E37">
+        <v>8</v>
+      </c>
+      <c r="F37" t="str">
+        <v>f901a74de1fd96ae6f1aef0b8319e4eddb2d5773</v>
+      </c>
+      <c r="G37" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G38" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Merge branch 'insure/develop' into insure2.0/secureInvest</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Integrate SecureInvest Features</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E39">
+        <v>1.33</v>
+      </c>
+      <c r="F39" t="str">
+        <v>2a9d947cbe273fdd8e5c29493bf41b378d660dec</v>
+      </c>
+      <c r="G39" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="B40" t="str">
+        <v>add</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Add Environment and Payment Gateway Configuration</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E40">
+        <v>2.67</v>
+      </c>
+      <c r="F40" t="str">
+        <v>375c93478bef64cdb7e9a780bb6d1e68c1109902</v>
+      </c>
+      <c r="G40" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="B41" t="str">
+        <v>add</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Implement Developer Console Component</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E41">
+        <v>2.67</v>
+      </c>
+      <c r="F41" t="str">
+        <v>4d0fd3607c349a8d69f17422ad68d36d3b26ded0</v>
+      </c>
+      <c r="G41" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="B42" t="str">
+        <v>secureInvest-riderAdded</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Enhance Secure Invest Options</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E42">
+        <v>1.33</v>
+      </c>
+      <c r="F42" t="str">
+        <v>fefbe626c36732b9363c5c98c9df68475c3c8b1e</v>
+      </c>
+      <c r="G42" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-04-21</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G43" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2026-04-21</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Merge branch 'insure2.0/secureInvest' into insure/develop</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Integrate Secure Investment Module</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E44">
+        <v>2.67</v>
+      </c>
+      <c r="F44" t="str">
+        <v>c5df19fe41804cdc3a3ff2963d46f5c0f501b4a5</v>
+      </c>
+      <c r="G44" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2026-04-21</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/ISNP into insure2.0/secureInvest</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Integrate ENACH Gateway URL and Validation Changes</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E45">
+        <v>5.33</v>
+      </c>
+      <c r="F45" t="str">
+        <v>9cb71c2bd2454fa93d6f415e877ad67970359b59</v>
+      </c>
+      <c r="G45" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G46" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Integrate OTP Verification Features</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E47">
+        <v>1.1</v>
+      </c>
+      <c r="F47" t="str">
+        <v>c098251634c57c548d527009d84b43ec1704ba41</v>
+      </c>
+      <c r="G47" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B48" t="str">
+        <v>fix: sync package-lock with package.json</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Synchronize package-lock with package.json</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E48">
+        <v>0.28</v>
+      </c>
+      <c r="F48" t="str">
+        <v>d6dd30dc3c8303c114e9a2e62afbd6a30a3a969d</v>
+      </c>
+      <c r="G48" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B49" t="str">
+        <v>rider premium mapping</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Implement Rider Premium Mapping Helper Functions</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E49">
+        <v>1.1</v>
+      </c>
+      <c r="F49" t="str">
+        <v>303affc8a58d89cd5fa4a833ae47d83064bd0d1f</v>
+      </c>
+      <c r="G49" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B50" t="str">
+        <v>BI called with rider</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Enhance Rider Sections for NRI Customers</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E50">
+        <v>1.66</v>
+      </c>
+      <c r="F50" t="str">
         <v>89d26b23f16a15177efb879ae78d0305f26844f1</v>
       </c>
-      <c r="G20" t="str">
-        <v>insure/secureInvest2.0</v>
+      <c r="G50" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Merge remote-tracking branch 'origin/insure/develop' into infinityInsure2.0/uat</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Integrate Future Income Options with Conditions</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E51">
+        <v>1.1</v>
+      </c>
+      <c r="F51" t="str">
+        <v>43f10d2b9beb838916cbf7afcec976e44c0dd6d2</v>
+      </c>
+      <c r="G51" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Merge Development Branch into UAT</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E52">
+        <v>0.55</v>
+      </c>
+      <c r="F52" t="str">
+        <v>849cf949bca28d84224ba0b3cc804f6ea0685a2b</v>
+      </c>
+      <c r="G52" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B53" t="str">
+        <v>package json fix</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Package JSON Configuration Update</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E53">
+        <v>0.55</v>
+      </c>
+      <c r="F53" t="str">
+        <v>2704e1bc206feb7affebb6a2eb2df8c10ba0ea55</v>
+      </c>
+      <c r="G53" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B54" t="str">
+        <v>sync package.json issue</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Synchronize package.json Dependencies</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Bug Fix</v>
+      </c>
+      <c r="E54">
+        <v>0.55</v>
+      </c>
+      <c r="F54" t="str">
+        <v>c05a99adf2c8c7ff431706c387f79cc9e91fc4b4</v>
+      </c>
+      <c r="G54" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Integration of Develop Branch into UAT</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E55">
+        <v>1.11</v>
+      </c>
+      <c r="F55" t="str">
+        <v>775de01c66ec153067e5f50f94893531842dc9d1</v>
+      </c>
+      <c r="G55" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2026-04-23</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G56" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2026-04-23</v>
+      </c>
+      <c r="B57" t="str">
+        <v>secure invest as per new figma and rider</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Update Secure Invest to Figma Design</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E57">
+        <v>8</v>
+      </c>
+      <c r="F57" t="str">
+        <v>49534134e59ffde6855a2e83008ea0fc12a8c2e8</v>
+      </c>
+      <c r="G57" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G58" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Integrate Additional BI Features</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E59">
+        <v>1.5</v>
+      </c>
+      <c r="F59" t="str">
+        <v>9d6d7951dd8046a338c08410dc063fc31d11c4ca</v>
+      </c>
+      <c r="G59" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Merge branch 'insure/secureInvest2.0' into insure/develop</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Integrate Secure Investment Features</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+      <c r="F60" t="str">
+        <v>6267c3d021cec4802466306cd28e932a5d4ae6e3</v>
+      </c>
+      <c r="G60" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B61" t="str">
+        <v>feat: add biFooterTwoStep configuration and premium calculation button label to journeyssr.json</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Add BI Footer Configuration and Premium Button Label</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E61">
+        <v>1</v>
+      </c>
+      <c r="F61" t="str">
+        <v>1cc5cfe77d6de78050560abcd51304815328ca76</v>
+      </c>
+      <c r="G61" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Merge branch 'insure/secureInvest2.0' into insure/develop</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Integrate Secure Invest 2.0 Features</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62" t="str">
+        <v>96c521486a959f33abff7d96909b9c2d686af9e9</v>
+      </c>
+      <c r="G62" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Merge branch 'insure/develop' into insure/secureInvest2.0</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Integrate Address and Income Validations</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Integration/Merge</v>
+      </c>
+      <c r="E63">
+        <v>1.5</v>
+      </c>
+      <c r="F63" t="str">
+        <v>09d272a9675c9e868df0ed9c9af14b2c6ae46131</v>
+      </c>
+      <c r="G63" t="str">
+        <v>infinityInsure2.0/uat</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2026-04-24</v>
+      </c>
+      <c r="B64" t="str">
+        <v>feat: implement two-step BI footer with premium calculation and section persistence enhancements</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Implement Two-Step BI Footer Enhancements</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Feature</v>
+      </c>
+      <c r="E64">
+        <v>2</v>
+      </c>
+      <c r="F64" t="str">
+        <v>036534a3288671c0d089ad02950c2fe3dace2605</v>
+      </c>
+      <c r="G64" t="str">
+        <v>infinityInsure2.0/uat</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement dynamic .env reload and exclude merge commits from processing and logging logic
</commit_message>
<xml_diff>
--- a/redmine-logger/backend/user_data/lumiqshubh23/git_commits.xlsx
+++ b/redmine-logger/backend/user_data/lumiqshubh23/git_commits.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,7 +427,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-04-01</v>
+        <v>2026-06-01</v>
       </c>
       <c r="B2" t="str">
         <v>Daily Scrum Call</v>
@@ -453,267 +453,267 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-04-01</v>
+        <v>2026-06-01</v>
       </c>
       <c r="B3" t="str">
-        <v>Merge remote-tracking branch 'origin/CR-36689-backend' into uat-common-backend-1</v>
+        <v>DM-22984 deathcover factor in igf</v>
       </c>
       <c r="C3" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="E3" t="str">
-        <v>b45e6c1d56d0c7977c25dde43e5533c3473350cd</v>
+        <v>5033a821c6e25b95378953140ed14edca12d0e84</v>
       </c>
       <c r="F3" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G3" t="str">
-        <v>Update Document Option Logic</v>
+        <v>DM-22984 deathcover factor in igf</v>
       </c>
       <c r="H3" t="str">
-        <v>Update Document Option Logic</v>
+        <v>DM-22984 deathcover factor in igf</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-04-01</v>
+        <v>2026-06-01</v>
       </c>
       <c r="B4" t="str">
-        <v>LA=&gt;PR in proposal form</v>
+        <v>DM-23043</v>
       </c>
       <c r="C4" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="E4" t="str">
-        <v>9eacdfea71d2af341bf4d5f68ef3baa57f34a750</v>
+        <v>7772684e682945f39c9cd52d75cb5bdb0c27e994</v>
       </c>
       <c r="F4" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G4" t="str">
-        <v>Update Document Option from LA to PR</v>
+        <v>DM-23043</v>
       </c>
       <c r="H4" t="str">
-        <v>Update Document Option from LA to PR</v>
+        <v>DM-23043</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-04-02</v>
+        <v>2026-06-01</v>
       </c>
       <c r="B5" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest  continue button issue</v>
       </c>
       <c r="C5" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2.66</v>
       </c>
       <c r="E5" t="str">
-        <v>N/A</v>
+        <v>d1b7e2f9d0fc330e4ec7fbf4b0baf95ef0b0f544</v>
       </c>
       <c r="F5" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G5" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest  continue button issue</v>
       </c>
       <c r="H5" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest  continue button issue</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-04-02</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B6" t="str">
-        <v>Merge branch 'CR-36689-backend' into uat-common-backend-1</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C6" t="str">
-        <v>Integration/Merge</v>
+        <v>Meeting</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>c13893e09868c8e55a880da96b2d1c8ed842bd12</v>
+        <v>N/A</v>
       </c>
       <c r="F6" t="str">
-        <v>uat-common-backend-1</v>
+        <v>N/A</v>
       </c>
       <c r="G6" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H6" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-04-02</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B7" t="str">
-        <v>proposal form photo</v>
+        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
       </c>
       <c r="C7" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D7">
-        <v>4</v>
+        <v>1.33</v>
       </c>
       <c r="E7" t="str">
-        <v>728198965083920c53df98ecd079c966f9582b55</v>
+        <v>09c6c080804f72a8df6c44653f478851330fccd8</v>
       </c>
       <c r="F7" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G7" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
       </c>
       <c r="H7" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-04-06</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B8" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
       </c>
       <c r="C8" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>1.33</v>
       </c>
       <c r="E8" t="str">
-        <v>N/A</v>
+        <v>15bd27fe6965ad8aa560d25a8a9f8c20cb5f1dd4</v>
       </c>
       <c r="F8" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G8" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
       </c>
       <c r="H8" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-04-06</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B9" t="str">
-        <v>rename route for insure2</v>
+        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
       </c>
       <c r="C9" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D9">
-        <v>1.6</v>
+        <v>1.33</v>
       </c>
       <c r="E9" t="str">
-        <v>69c09dbd6ddc08e72e384b683c0dd09f64f36272</v>
+        <v>eb7cf33323d4a62471b0bbea27611f71d129673d</v>
       </c>
       <c r="F9" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G9" t="str">
-        <v>Refactor TPA Route and Add GA Check</v>
+        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
       </c>
       <c r="H9" t="str">
-        <v>Refactor TPA Route and Add GA Check</v>
+        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-04-06</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B10" t="str">
-        <v>make pan wrapper generic</v>
+        <v>DM-23070 Pincode api run after clicking outside the field</v>
       </c>
       <c r="C10" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D10">
-        <v>1.6</v>
+        <v>1.33</v>
       </c>
       <c r="E10" t="str">
-        <v>109771a04b7823cb8b195828bfe51e7acc4e77d5</v>
+        <v>45239ff3a1193cb91d9b366fda2e615d55aaf5ed</v>
       </c>
       <c r="F10" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G10" t="str">
-        <v>Make Axios Wrapper Generic</v>
+        <v>DM-23070 Pincode api run after clicking outside the field</v>
       </c>
       <c r="H10" t="str">
-        <v>Make Axios Wrapper Generic</v>
+        <v>DM-23070 Pincode api run after clicking outside the field</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-04-06</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B11" t="str">
-        <v>generic wrapper</v>
+        <v>secure Invest afr fix</v>
       </c>
       <c r="C11" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D11">
-        <v>3.2</v>
+        <v>1.33</v>
       </c>
       <c r="E11" t="str">
-        <v>0db337c779bb5b41c01d6792d5a89d2164677964</v>
+        <v>38d50b8f7fac49f9b16d29c8582958bbb40ae9ff</v>
       </c>
       <c r="F11" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G11" t="str">
-        <v>Implement Axios Request Wrapper</v>
+        <v>secure Invest afr fix</v>
       </c>
       <c r="H11" t="str">
-        <v>Implement Axios Request Wrapper</v>
+        <v>secure Invest afr fix</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-04-06</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B12" t="str">
-        <v>new routes for ISNP2.0</v>
+        <v>secure Invest afr fix</v>
       </c>
       <c r="C12" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D12">
-        <v>1.6</v>
+        <v>1.35</v>
       </c>
       <c r="E12" t="str">
-        <v>46369462a4a27be7e4a52103b3ea980ad7d1bde8</v>
+        <v>5e4a4a77c57a009e00e9661f54a8f2b620d3e266</v>
       </c>
       <c r="F12" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G12" t="str">
-        <v>Implement New ISNP 2.0 Routes</v>
+        <v>secure Invest afr fix</v>
       </c>
       <c r="H12" t="str">
-        <v>Implement New ISNP 2.0 Routes</v>
+        <v>secure Invest afr fix</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-04-07</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B13" t="str">
         <v>Daily Scrum Call</v>
@@ -739,813 +739,813 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-04-07</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B14" t="str">
-        <v>Merge branch 'insure-api-wrapper' of https://github.com/lumiqai/isnp-backend-v2 into insure-api-wrapper</v>
+        <v>Revert "alternative number added"</v>
       </c>
       <c r="C14" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D14">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="E14" t="str">
-        <v>f135d9f9bf66647b7227ceeddd7c064bfe0dd9f4</v>
+        <v>60606c0a103f76c72422f3155668650136edcd40</v>
       </c>
       <c r="F14" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G14" t="str">
-        <v>Add CIBIL Insurance Insights API Endpoint</v>
+        <v>Revert "alternative number added"</v>
       </c>
       <c r="H14" t="str">
-        <v>Add CIBIL Insurance Insights API Endpoint</v>
+        <v>Revert "alternative number added"</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-04-07</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B15" t="str">
-        <v>retailduplicateApplicationNumber</v>
+        <v>alternative number added</v>
       </c>
       <c r="C15" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D15">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="E15" t="str">
-        <v>6b42e2097e52b2fc8bca0b8369923e986ee4fa4f</v>
+        <v>370237486317451707c49b64a237b56148ad9bc7</v>
       </c>
       <c r="F15" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G15" t="str">
-        <v>Implement Retail App Number Duplicate Check</v>
+        <v>alternative number added</v>
       </c>
       <c r="H15" t="str">
-        <v>Implement Retail App Number Duplicate Check</v>
+        <v>alternative number added</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-04-07</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B16" t="str">
-        <v>application number exist api</v>
+        <v>rop error msg fix</v>
       </c>
       <c r="C16" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D16">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="E16" t="str">
-        <v>61672101b8bc72d019e4194c25c8471a8eb7db00</v>
+        <v>b37bc9ee06f2575abaa1113396367f1ac801bdff</v>
       </c>
       <c r="F16" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G16" t="str">
-        <v>Implement Application Number Existence Check API</v>
+        <v>rop error msg fix</v>
       </c>
       <c r="H16" t="str">
-        <v>Implement Application Number Existence Check API</v>
+        <v>rop error msg fix</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-04-14</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B17" t="str">
-        <v>Daily Scrum Call</v>
+        <v>wealth edge fund issue fix</v>
       </c>
       <c r="C17" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" t="str">
-        <v>N/A</v>
+        <v>a3c9496d6ae1e5d5bed1bff81002ff7360c4d36a</v>
       </c>
       <c r="F17" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G17" t="str">
-        <v>Daily Scrum Call</v>
+        <v>wealth edge fund issue fix</v>
       </c>
       <c r="H17" t="str">
-        <v>Daily Scrum Call</v>
+        <v>wealth edge fund issue fix</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-04-14</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B18" t="str">
-        <v>change in fm and rm</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C18" t="str">
-        <v>Refactor</v>
+        <v>Meeting</v>
       </c>
       <c r="D18">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v>d9abbb744e8db8ed76923c3097a01bad0d6611fb</v>
+        <v>N/A</v>
       </c>
       <c r="F18" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G18" t="str">
-        <v>Refactor Address Handling in Mapper</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H18" t="str">
-        <v>Refactor Address Handling in Mapper</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-04-16</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B19" t="str">
-        <v>Daily Scrum Call</v>
+        <v>spelling mistake fix</v>
       </c>
       <c r="C19" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="E19" t="str">
-        <v>N/A</v>
+        <v>4a829a71dfd645d746a114dcaeabd3646dfd11f4</v>
       </c>
       <c r="F19" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G19" t="str">
-        <v>Daily Scrum Call</v>
+        <v>spelling mistake fix</v>
       </c>
       <c r="H19" t="str">
-        <v>Daily Scrum Call</v>
+        <v>spelling mistake fix</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-04-16</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B20" t="str">
-        <v>Merge branch 'ISNP2.0-viewDoc' into insure/develop</v>
+        <v>mariner field issue</v>
       </c>
       <c r="C20" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D20">
-        <v>2.29</v>
+        <v>1.14</v>
       </c>
       <c r="E20" t="str">
-        <v>97ec690b39cc3d63bf6f87d850cd6d0c165ef92e</v>
+        <v>6f8e7ceed8731e893cf5fc9d2577123d8cd996f3</v>
       </c>
       <c r="F20" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G20" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>mariner field issue</v>
       </c>
       <c r="H20" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>mariner field issue</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-04-16</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B21" t="str">
-        <v>view doc</v>
+        <v>wealth edge continue issue fix</v>
       </c>
       <c r="C21" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D21">
-        <v>2.29</v>
+        <v>1.14</v>
       </c>
       <c r="E21" t="str">
-        <v>d8ba6ebbed9e1c2488d60aa58f94bd2b07b09bca</v>
+        <v>76bc99847e8c16318d11785e10b6e8abc52001c1</v>
       </c>
       <c r="F21" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G21" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>wealth edge continue issue fix</v>
       </c>
       <c r="H21" t="str">
-        <v>Enhance Document Retrieval Logic</v>
+        <v>wealth edge continue issue fix</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-04-16</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B22" t="str">
-        <v>Merge branch 'insure/develop' into uat-common-backend-1</v>
+        <v>bi pdf through sms</v>
       </c>
       <c r="C22" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D22">
-        <v>3.42</v>
+        <v>1.14</v>
       </c>
       <c r="E22" t="str">
-        <v>569367c297664fb8166da5ce886645b0f91f7a07</v>
+        <v>af1fabf41c1901c58a4535fe6c49933536afed1c</v>
       </c>
       <c r="F22" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G22" t="str">
-        <v>Integrate New Features and Address Changes</v>
+        <v>bi pdf through sms</v>
       </c>
       <c r="H22" t="str">
-        <v>Integrate New Features and Address Changes</v>
+        <v>bi pdf through sms</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B23" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23175</v>
       </c>
       <c r="C23" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="E23" t="str">
-        <v>N/A</v>
+        <v>0dd43a17d6c491ce1212b63b140285018b28922e</v>
       </c>
       <c r="F23" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G23" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23175</v>
       </c>
       <c r="H23" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23175</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B24" t="str">
-        <v>rider</v>
+        <v>DM-22975 illitrate mapping</v>
       </c>
       <c r="C24" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="E24" t="str">
-        <v>ede8eb520f4c961d93e1beb93bd5f1a6d550e59a</v>
+        <v>cbaaa9fedfb48e753e7ee7c11737ea9887fb225f</v>
       </c>
       <c r="F24" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G24" t="str">
-        <v>Enhance Payload Structure for Riders Section</v>
+        <v>DM-22975 illitrate mapping</v>
       </c>
       <c r="H24" t="str">
-        <v>Enhance Payload Structure for Riders Section</v>
+        <v>DM-22975 illitrate mapping</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B25" t="str">
-        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/isnp-backend-v2 into insure/develop-secureInvest</v>
+        <v>address flow chnage</v>
       </c>
       <c r="C25" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>1.16</v>
       </c>
       <c r="E25" t="str">
-        <v>45d4634821af87947066c149ca21aa31b6621fa0</v>
+        <v>bbca155bf05e640939b18486d9a0e0b20f7cf62e</v>
       </c>
       <c r="F25" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G25" t="str">
-        <v>Merge Develop Branch into SecureInvest</v>
+        <v>address flow chnage</v>
       </c>
       <c r="H25" t="str">
-        <v>Merge Develop Branch into SecureInvest</v>
+        <v>address flow chnage</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B26" t="str">
-        <v>secure invest fm</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C26" t="str">
-        <v>Feature</v>
+        <v>Meeting</v>
       </c>
       <c r="D26">
         <v>1</v>
       </c>
       <c r="E26" t="str">
-        <v>a89468656c7621660f6b4b7379bed5386837ffb2</v>
+        <v>N/A</v>
       </c>
       <c r="F26" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G26" t="str">
-        <v>Enhance Secure Invest Payload Handling</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H26" t="str">
-        <v>Enhance Secure Invest Payload Handling</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B27" t="str">
-        <v>Merge remote-tracking branch 'origin/insure/develop' into insure/develop-secureInvest</v>
+        <v>secure invest sto fund logic</v>
       </c>
       <c r="C27" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E27" t="str">
-        <v>a9583a2ecf639e9ac90c5f8470f6d5fd0c61e2b7</v>
+        <v>0f8491441ef27c57ea6a99411132fb25e32eda21</v>
       </c>
       <c r="F27" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G27" t="str">
-        <v>Integrate Fetch Insure Journeys Controller</v>
+        <v>secure invest sto fund logic</v>
       </c>
       <c r="H27" t="str">
-        <v>Integrate Fetch Insure Journeys Controller</v>
+        <v>secure invest sto fund logic</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B28" t="str">
-        <v>generate bi api integartion and fallback of fund alloction</v>
+        <v>Revert "DM-23121 if single option then autoSelect"</v>
       </c>
       <c r="C28" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E28" t="str">
-        <v>61591ff20a5c467ab4105ce52a4240641099a7cb</v>
+        <v>298c2849370ac0d64d6c362b14e9ebdb63501646</v>
       </c>
       <c r="F28" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G28" t="str">
-        <v>Implement BI API Integration for Fund Allocation</v>
+        <v>Revert "DM-23121 if single option then autoSelect"</v>
       </c>
       <c r="H28" t="str">
-        <v>Implement BI API Integration for Fund Allocation</v>
+        <v>Revert "DM-23121 if single option then autoSelect"</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-04-21</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B29" t="str">
-        <v>Merge branch 'insure/develop-secureInvest' into uat-common-backend-1</v>
+        <v>aadhar masked when 12 diigit</v>
       </c>
       <c r="C29" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D29">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E29" t="str">
-        <v>b5b79f292f5a0c249f65f734dd2796ad0c7604bf</v>
+        <v>42e680234bb7454719e3e454aa541d9cda441ab4</v>
       </c>
       <c r="F29" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G29" t="str">
-        <v>Integrate Secure Investment Features</v>
+        <v>aadhar masked when 12 diigit</v>
       </c>
       <c r="H29" t="str">
-        <v>Integrate Secure Investment Features</v>
+        <v>aadhar masked when 12 diigit</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-04-22</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B30" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="C30" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E30" t="str">
-        <v>N/A</v>
+        <v>093f9840d78111faaa0b8ba1bc26b576dd7b76ac</v>
       </c>
       <c r="F30" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G30" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="H30" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-04-22</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B31" t="str">
-        <v>Merge branch 'insure/develop' into insure/develop-secureInvest</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="C31" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D31">
         <v>1.6</v>
       </c>
       <c r="E31" t="str">
-        <v>29617eca1699b26755189e146880659da0bc370e</v>
+        <v>696502680c74817d742c55d8828822a6980de037</v>
       </c>
       <c r="F31" t="str">
-        <v>insure/develop</v>
+        <v>infinityInsure2.0/uat</v>
       </c>
       <c r="G31" t="str">
-        <v>Integrate Secure Investment Enhancements</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="H31" t="str">
-        <v>Integrate Secure Investment Enhancements</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-04-22</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B32" t="str">
-        <v>controller fix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C32" t="str">
-        <v>Refactor</v>
+        <v>Meeting</v>
       </c>
       <c r="D32">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E32" t="str">
-        <v>76508113b337667e04ece59528f7823a2e0aefb9</v>
+        <v>N/A</v>
       </c>
       <c r="F32" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G32" t="str">
-        <v>Improve BI Payload Builder Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H32" t="str">
-        <v>Improve BI Payload Builder Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-04-22</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B33" t="str">
-        <v>Merge branch 'insure/develop-secureInvest' into insure/develop</v>
+        <v>secure invest not fund auto select</v>
       </c>
       <c r="C33" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D33">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="E33" t="str">
-        <v>0799be42e81755c2a0c36b23719a4602ca426cc5</v>
+        <v>39fd1833bc250a89717977e1e3283d43130b3287</v>
       </c>
       <c r="F33" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G33" t="str">
-        <v>Integrate Secure Investment Features</v>
+        <v>secure invest not fund auto select</v>
       </c>
       <c r="H33" t="str">
-        <v>Integrate Secure Investment Features</v>
+        <v>secure invest not fund auto select</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-04-22</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B34" t="str">
-        <v>Merge remote-tracking branch 'origin/insure/develop' into uat-common-backend-1</v>
+        <v>annur wealth edge issue fix</v>
       </c>
       <c r="C34" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D34">
-        <v>1.6</v>
+        <v>4</v>
       </c>
       <c r="E34" t="str">
-        <v>39381a458ce3958ff554d723dc76d18df7395d9b</v>
+        <v>50f6c88d2c7fbab5c57efaa5723a34b71f4386a0</v>
       </c>
       <c r="F34" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G34" t="str">
-        <v>Integrate Insure BI Payload Changes</v>
+        <v>annur wealth edge issue fix</v>
       </c>
       <c r="H34" t="str">
-        <v>Integrate Insure BI Payload Changes</v>
+        <v>annur wealth edge issue fix</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-04-22</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B35" t="str">
-        <v>Merge remote-tracking branch 'origin/insure/develop' into uat-common-backend-1</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C35" t="str">
-        <v>Integration/Merge</v>
+        <v>Meeting</v>
       </c>
       <c r="D35">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E35" t="str">
-        <v>494058cef7c631033cb8cf0154b25c5b6ac01928</v>
+        <v>N/A</v>
       </c>
       <c r="F35" t="str">
-        <v>uat-common-backend-1</v>
+        <v>N/A</v>
       </c>
       <c r="G35" t="str">
-        <v>Integrate Develop Branch into UAT</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H35" t="str">
-        <v>Integrate Develop Branch into UAT</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-04-24</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B36" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest liquide fund issue fix</v>
       </c>
       <c r="C36" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E36" t="str">
-        <v>N/A</v>
+        <v>db04074e51693acf46994b47b89ae6221301b597</v>
       </c>
       <c r="F36" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G36" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest liquide fund issue fix</v>
       </c>
       <c r="H36" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest liquide fund issue fix</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-04-24</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B37" t="str">
-        <v>Merge branch 'insure/develop-secureInvest' into insure/develop</v>
+        <v>secureInvest whole life option</v>
       </c>
       <c r="C37" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D37">
-        <v>2.13</v>
+        <v>4</v>
       </c>
       <c r="E37" t="str">
-        <v>b76a88fdaabee2ff38a2fa37f471617d2d6bdcee</v>
+        <v>01fb61970864ac23e69baf11116af08bba99c552</v>
       </c>
       <c r="F37" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G37" t="str">
-        <v>Integrate Secure Investment Features</v>
+        <v>secureInvest whole life option</v>
       </c>
       <c r="H37" t="str">
-        <v>Integrate Secure Investment Features</v>
+        <v>secureInvest whole life option</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-04-24</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B38" t="str">
-        <v>feat: enhance INSURE application mapping with section merging and rider code normalization</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C38" t="str">
-        <v>Feature</v>
+        <v>Meeting</v>
       </c>
       <c r="D38">
-        <v>2.13</v>
+        <v>1</v>
       </c>
       <c r="E38" t="str">
-        <v>aae189ade9eb77b37b4a203186ed45f862c7ffe3</v>
+        <v>N/A</v>
       </c>
       <c r="F38" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G38" t="str">
-        <v>Enhance INSURE Application Mapping Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H38" t="str">
-        <v>Enhance INSURE Application Mapping Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-04-24</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B39" t="str">
-        <v>Merge branch 'insure/develop' into insure/develop-secureInvest</v>
+        <v>uncheck dob feature</v>
       </c>
       <c r="C39" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D39">
-        <v>2.13</v>
+        <v>1.33</v>
       </c>
       <c r="E39" t="str">
-        <v>7d1d79604cc654021d82bbd25d477cf72fc21f43</v>
+        <v>ead293f3b06815288e7967a7bb7e52107e7f6c94</v>
       </c>
       <c r="F39" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G39" t="str">
-        <v>Integrate Spouse Questionnaire Features</v>
+        <v>uncheck dob feature</v>
       </c>
       <c r="H39" t="str">
-        <v>Integrate Spouse Questionnaire Features</v>
+        <v>uncheck dob feature</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-04-24</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B40" t="str">
-        <v>Merge branch 'insure/develop' into uat-common-backend-1</v>
+        <v>adress flow change by enhancement</v>
       </c>
       <c r="C40" t="str">
-        <v>Integration/Merge</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D40">
-        <v>1.61</v>
+        <v>1.33</v>
       </c>
       <c r="E40" t="str">
-        <v>e0025b7e51a13b891bced559a2c18c9b89556658</v>
+        <v>3097285a98b6d6a00da498f480f76072c6e1c592</v>
       </c>
       <c r="F40" t="str">
-        <v>uat-common-backend-1</v>
+        <v>insure/develop</v>
       </c>
       <c r="G40" t="str">
-        <v>Integrate FNA Section Merging Logic</v>
+        <v>adress flow change by enhancement</v>
       </c>
       <c r="H40" t="str">
-        <v>Integrate FNA Section Merging Logic</v>
+        <v>adress flow change by enhancement</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-05-04</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B41" t="str">
-        <v>Daily Scrum Call</v>
+        <v>address enhanacement</v>
       </c>
       <c r="C41" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>1.33</v>
       </c>
       <c r="E41" t="str">
-        <v>N/A</v>
+        <v>1df15fe16d18561d9ae557d4af7f483a2d1939df</v>
       </c>
       <c r="F41" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G41" t="str">
-        <v>Daily Scrum Call</v>
+        <v>address enhanacement</v>
       </c>
       <c r="H41" t="str">
-        <v>Daily Scrum Call</v>
+        <v>address enhanacement</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-05-04</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B42" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>annur navigate to next even if api fail</v>
       </c>
       <c r="C42" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D42">
-        <v>2.67</v>
+        <v>1.33</v>
       </c>
       <c r="E42" t="str">
-        <v>d9f4b6d07b8e49dcb269b4671ab5c2bbe942329d</v>
+        <v>c7f0f41075db3410129cceeaf5f971b6c742e667</v>
       </c>
       <c r="F42" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G42" t="str">
-        <v>Update Secure Invest Riders Section</v>
+        <v>annur navigate to next even if api fail</v>
       </c>
       <c r="H42" t="str">
-        <v>Update Secure Invest Riders Section</v>
+        <v>annur navigate to next even if api fail</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-05-04</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B43" t="str">
-        <v>Merge branch 'insure/wealthEdge' into insure/develop</v>
+        <v>add speical character validation on address</v>
       </c>
       <c r="C43" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D43">
-        <v>2.67</v>
+        <v>1.33</v>
       </c>
       <c r="E43" t="str">
-        <v>691b6ae971f8d9be67fd4e68e0220215a9049246</v>
+        <v>a385b36d4af4fbaa692a2bb9c9b9d071bdf973d7</v>
       </c>
       <c r="F43" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G43" t="str">
-        <v>Enhance Secure Invest Riders Configuration</v>
+        <v>add speical character validation on address</v>
       </c>
       <c r="H43" t="str">
-        <v>Enhance Secure Invest Riders Configuration</v>
+        <v>add speical character validation on address</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-05-04</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B44" t="str">
-        <v>feat: update Secure Invest and Titanium riders configuration and validation logic</v>
+        <v>wealth edge issue fix</v>
       </c>
       <c r="C44" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D44">
-        <v>2.66</v>
+        <v>1.35</v>
       </c>
       <c r="E44" t="str">
-        <v>57db8a9a65b713e2e6f8835abbf050a8703011f4</v>
+        <v>ac9e7046f9f21089761a6d96c097f94bb0ed7165</v>
       </c>
       <c r="F44" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G44" t="str">
-        <v>Update Configuration and Validation Logic for Riders</v>
+        <v>wealth edge issue fix</v>
       </c>
       <c r="H44" t="str">
-        <v>Update Configuration and Validation Logic for Riders</v>
+        <v>wealth edge issue fix</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-05-07</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B45" t="str">
         <v>Daily Scrum Call</v>
@@ -1571,371 +1571,371 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-05-07</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B46" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
       </c>
       <c r="C46" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D46">
-        <v>3</v>
+        <v>1.14</v>
       </c>
       <c r="E46" t="str">
-        <v>5dba728b974386e382fec8fe5d70147242ae0e86</v>
+        <v>4f07e17fae2fa8cb32e3bf179b06b7e20fe8942f</v>
       </c>
       <c r="F46" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G46" t="str">
-        <v>Enhance Product Details Section Layout</v>
+        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
       </c>
       <c r="H46" t="str">
-        <v>Enhance Product Details Section Layout</v>
+        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-05-07</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B47" t="str">
-        <v>Merge branch 'insure/IGFP' into insure/develop</v>
+        <v>pan number must be 10</v>
       </c>
       <c r="C47" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D47">
-        <v>2</v>
+        <v>1.14</v>
       </c>
       <c r="E47" t="str">
-        <v>a178806adc4345fcde9b28a746e02da6a0b28e57</v>
+        <v>6cf0060bb8f1341fd076662f36f21ea3ff1bf2e5</v>
       </c>
       <c r="F47" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G47" t="str">
-        <v>Implement IGFP Product Details Section</v>
+        <v>pan number must be 10</v>
       </c>
       <c r="H47" t="str">
-        <v>Implement IGFP Product Details Section</v>
+        <v>pan number must be 10</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-05-07</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B48" t="str">
-        <v>igf development</v>
+        <v>Relationship with PEP other field add</v>
       </c>
       <c r="C48" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D48">
-        <v>3</v>
+        <v>1.14</v>
       </c>
       <c r="E48" t="str">
-        <v>bdfe068cdd05d50fb3cd1794e5fb6285aafb318c</v>
+        <v>37de77bf0a1c9579237aa77cced98d5f64dfd18c</v>
       </c>
       <c r="F48" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G48" t="str">
-        <v>Implement IGFP Product Details Section</v>
+        <v>Relationship with PEP other field add</v>
       </c>
       <c r="H48" t="str">
-        <v>Implement IGFP Product Details Section</v>
+        <v>Relationship with PEP other field add</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-05-11</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B49" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
       </c>
       <c r="C49" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="E49" t="str">
-        <v>N/A</v>
+        <v>54688bbceecfe9edf3baff9717ace090b07f228f</v>
       </c>
       <c r="F49" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G49" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
       </c>
       <c r="H49" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-05-11</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B50" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>PO personal Health details should not come for form 2 cases</v>
       </c>
       <c r="C50" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D50">
-        <v>2</v>
+        <v>1.14</v>
       </c>
       <c r="E50" t="str">
-        <v>6bfbdf4e81a1896faf73f645beacbcca7a6e54c2</v>
+        <v>d9b9549bf78158a844a9ce66cea71510c9ba251b</v>
       </c>
       <c r="F50" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G50" t="str">
-        <v>Enhance Secure Investment Plan Options</v>
+        <v>PO personal Health details should not come for form 2 cases</v>
       </c>
       <c r="H50" t="str">
-        <v>Enhance Secure Investment Plan Options</v>
+        <v>PO personal Health details should not come for form 2 cases</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-05-11</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B51" t="str">
-        <v>Merge branch 'insure/secureInvest-bugs' into insure/develop</v>
+        <v>for 2 case questionior handle</v>
       </c>
       <c r="C51" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D51">
-        <v>2</v>
+        <v>1.14</v>
       </c>
       <c r="E51" t="str">
-        <v>5fdc90e1cf1dca0283322d834f98050912414813</v>
+        <v>09fd7f027227956b052b1b960c1097944cb1a60f</v>
       </c>
       <c r="F51" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G51" t="str">
-        <v>Enhance Secure Investment Policy Options</v>
+        <v>for 2 case questionior handle</v>
       </c>
       <c r="H51" t="str">
-        <v>Enhance Secure Investment Policy Options</v>
+        <v>for 2 case questionior handle</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-05-11</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B52" t="str">
-        <v>secure invest bugs fixes</v>
+        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
       </c>
       <c r="C52" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D52">
-        <v>2</v>
+        <v>1.16</v>
       </c>
       <c r="E52" t="str">
-        <v>7e9049f57094ad621d732c8febb40cb944a63706</v>
+        <v>cb4c27537d4c9ac33488c2d2d3ced67deb1ff4d8</v>
       </c>
       <c r="F52" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G52" t="str">
-        <v>Enhance Secure Investment Policies</v>
+        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
       </c>
       <c r="H52" t="str">
-        <v>Enhance Secure Investment Policies</v>
+        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-05-11</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B53" t="str">
-        <v>p4gplus development intial setup</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C53" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" t="str">
-        <v>8820894ac83ed6075c2951ea22d5f1a5c8749ded</v>
+        <v>N/A</v>
       </c>
       <c r="F53" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G53" t="str">
-        <v>Setup Initial Framework for Promise4GrowthPlus</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H53" t="str">
-        <v>Setup Initial Framework for Promise4GrowthPlus</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-05-12</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B54" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-2394</v>
       </c>
       <c r="C54" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>1.33</v>
       </c>
       <c r="E54" t="str">
-        <v>N/A</v>
+        <v>a5ee1019cdcb541ec627f383ab6c9104045f048c</v>
       </c>
       <c r="F54" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G54" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-2394</v>
       </c>
       <c r="H54" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-2394</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-05-12</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B55" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>upload checkbox feature</v>
       </c>
       <c r="C55" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D55">
-        <v>2.67</v>
+        <v>1.33</v>
       </c>
       <c r="E55" t="str">
-        <v>0373dcf55c64c18a69f461d8b94565e4c99d7074</v>
+        <v>b502a004028755e9856792303ca1f5e33726b8a2</v>
       </c>
       <c r="F55" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G55" t="str">
-        <v>Enhance Choose Funds Section Functionality</v>
+        <v>upload checkbox feature</v>
       </c>
       <c r="H55" t="str">
-        <v>Enhance Choose Funds Section Functionality</v>
+        <v>upload checkbox feature</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-05-12</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B56" t="str">
-        <v>Merge branch 'insure/wealthEdge-bugs' into insure/develop</v>
+        <v>Revert "address proof type also added"</v>
       </c>
       <c r="C56" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D56">
-        <v>2.67</v>
+        <v>1.33</v>
       </c>
       <c r="E56" t="str">
-        <v>dc522d336a93c8ead98f803d4d8698e066ab6337</v>
+        <v>7ba1767399890d1c2cde14e5b2a6a743e86392ff</v>
       </c>
       <c r="F56" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G56" t="str">
-        <v>Enhance Fund Details Integration</v>
+        <v>Revert "address proof type also added"</v>
       </c>
       <c r="H56" t="str">
-        <v>Enhance Fund Details Integration</v>
+        <v>Revert "address proof type also added"</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-05-12</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B57" t="str">
-        <v>wealthEdge bug fixed</v>
+        <v>address proof type also added</v>
       </c>
       <c r="C57" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D57">
-        <v>2.66</v>
+        <v>1.33</v>
       </c>
       <c r="E57" t="str">
-        <v>bfd46e81f4acfc7996844c2bbf662726ec1f1e46</v>
+        <v>62940a6c9d80db350938204b6164a4210a6329ca</v>
       </c>
       <c r="F57" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G57" t="str">
-        <v>Enhance Fund Selection Logic in Wealth Edge</v>
+        <v>address proof type also added</v>
       </c>
       <c r="H57" t="str">
-        <v>Enhance Fund Selection Logic in Wealth Edge</v>
+        <v>address proof type also added</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-05-13</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B58" t="str">
-        <v>Daily Scrum Call</v>
+        <v>annur api fail navigateion</v>
       </c>
       <c r="C58" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>1.33</v>
       </c>
       <c r="E58" t="str">
-        <v>N/A</v>
+        <v>ca7fe937e633709130fcf2b62edc7582dd30f9f6</v>
       </c>
       <c r="F58" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G58" t="str">
-        <v>Daily Scrum Call</v>
+        <v>annur api fail navigateion</v>
       </c>
       <c r="H58" t="str">
-        <v>Daily Scrum Call</v>
+        <v>annur api fail navigateion</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-05-13</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B59" t="str">
-        <v>Merge branch 'insure/develop' into insure/P4Gplus</v>
+        <v>add age proof as per DM-23374</v>
       </c>
       <c r="C59" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D59">
-        <v>8</v>
+        <v>1.35</v>
       </c>
       <c r="E59" t="str">
-        <v>4364fcfdb0d8409505cf001d0dede8cee3a121b2</v>
+        <v>56f5281030fca42a747e2a596def58064e93f69e</v>
       </c>
       <c r="F59" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G59" t="str">
-        <v>Implement Offline Notification Component</v>
+        <v>add age proof as per DM-23374</v>
       </c>
       <c r="H59" t="str">
-        <v>Implement Offline Notification Component</v>
+        <v>add age proof as per DM-23374</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-05-14</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B60" t="str">
         <v>Daily Scrum Call</v>
@@ -1961,1203 +1961,891 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-05-14</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B61" t="str">
-        <v>Merge remote-tracking branch 'origin/insure/develop' into infinityInsure2.0/uat</v>
+        <v>Dm-23443</v>
       </c>
       <c r="C61" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D61">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="E61" t="str">
-        <v>f6990533bfbff6efdcdf8458e628887304e1c506</v>
+        <v>f2fe5fcd220af0cf8bd4bc27899735ade613a321</v>
       </c>
       <c r="F61" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G61" t="str">
-        <v>Enhance Promise4GrowthPlus Product Details</v>
+        <v>Dm-23443</v>
       </c>
       <c r="H61" t="str">
-        <v>Enhance Promise4GrowthPlus Product Details</v>
+        <v>Dm-23443</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-05-14</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B62" t="str">
-        <v>Merge branch 'insure/P4Gplus' into insure/develop</v>
+        <v>DM-23381</v>
       </c>
       <c r="C62" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D62">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="E62" t="str">
-        <v>97f1082671b7e76c7c226cc3dd9a22f9d1854573</v>
+        <v>ff9fd4f1691ccfc490c3d03f1c0095e68eefc42b</v>
       </c>
       <c r="F62" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G62" t="str">
-        <v>Add Promise 4 Growth Plus Product Details</v>
+        <v>DM-23381</v>
       </c>
       <c r="H62" t="str">
-        <v>Add Promise 4 Growth Plus Product Details</v>
+        <v>DM-23381</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-05-14</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B63" t="str">
-        <v>Merge remote-tracking branch 'origin/insure/develop' into insure/P4Gplus</v>
+        <v>pan validation error msg</v>
       </c>
       <c r="C63" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D63">
         <v>1.6</v>
       </c>
       <c r="E63" t="str">
-        <v>f8034c6d804460be9a47747cc3e570b327cfd50a</v>
+        <v>d5a54a5cd7a0774aaf5d181e53979f5098e26522</v>
       </c>
       <c r="F63" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G63" t="str">
-        <v>Enhance Form Builder and PDF Library Integration</v>
+        <v>pan validation error msg</v>
       </c>
       <c r="H63" t="str">
-        <v>Enhance Form Builder and PDF Library Integration</v>
+        <v>pan validation error msg</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-05-14</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B64" t="str">
-        <v>Promise4growth plus development of BI and unified launch</v>
+        <v>Non - School Going Child have value 185</v>
       </c>
       <c r="C64" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D64">
         <v>1.6</v>
       </c>
       <c r="E64" t="str">
-        <v>025508b8be84e9127d10e3fdb4754cc497d94cac</v>
+        <v>25c68f96763134e98d0a9ea38a91c154157a7cfa</v>
       </c>
       <c r="F64" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G64" t="str">
-        <v>Enhance BI Features for Policy Options</v>
+        <v>Non - School Going Child have value 185</v>
       </c>
       <c r="H64" t="str">
-        <v>Enhance BI Features for Policy Options</v>
+        <v>Non - School Going Child have value 185</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-05-15</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B65" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Dm-23443</v>
       </c>
       <c r="C65" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D65">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E65" t="str">
-        <v>N/A</v>
+        <v>3e07715dfd25da43ca278839e96c01e446ef161a</v>
       </c>
       <c r="F65" t="str">
-        <v>N/A</v>
+        <v>infinityInsure2.0/uat</v>
       </c>
       <c r="G65" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Dm-23443</v>
       </c>
       <c r="H65" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Dm-23443</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-05-15</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B66" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C66" t="str">
-        <v>Bug Fix</v>
+        <v>Meeting</v>
       </c>
       <c r="D66">
-        <v>4.57</v>
+        <v>1</v>
       </c>
       <c r="E66" t="str">
-        <v>ffa76336bc0bd7de7c10eef661fa7d3766deb332</v>
+        <v>N/A</v>
       </c>
       <c r="F66" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G66" t="str">
-        <v>Improve Input Field Validation Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H66" t="str">
-        <v>Improve Input Field Validation Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-05-15</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B67" t="str">
-        <v>secureInvest and WE bug fix</v>
+        <v>address checkbox fix</v>
       </c>
       <c r="C67" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D67">
-        <v>3.43</v>
+        <v>4</v>
       </c>
       <c r="E67" t="str">
-        <v>40e9570f9cf0faf6600f36089d0e13bfcab97b87</v>
+        <v>407858e401bc2975e70bdf5856f6ab9b140f0960</v>
       </c>
       <c r="F67" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G67" t="str">
-        <v>Fix Input Validation and Synchronization Logic</v>
+        <v>address checkbox fix</v>
       </c>
       <c r="H67" t="str">
-        <v>Fix Input Validation and Synchronization Logic</v>
+        <v>address checkbox fix</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B68" t="str">
-        <v>Daily Scrum Call</v>
+        <v>add address proof type</v>
       </c>
       <c r="C68" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D68">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E68" t="str">
-        <v>N/A</v>
+        <v>bdb0ea1853713cfe111eda9c06d8564bea6c2b79</v>
       </c>
       <c r="F68" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G68" t="str">
-        <v>Daily Scrum Call</v>
+        <v>add address proof type</v>
       </c>
       <c r="H68" t="str">
-        <v>Daily Scrum Call</v>
+        <v>add address proof type</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-19</v>
       </c>
       <c r="B69" t="str">
-        <v>Merge pull request #1944 from lumiqai/fix/suitabilityMatrix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C69" t="str">
-        <v>Bug Fix</v>
+        <v>Meeting</v>
       </c>
       <c r="D69">
-        <v>0.62</v>
+        <v>1</v>
       </c>
       <c r="E69" t="str">
-        <v>aaeef24c498c03b9718e18e9e79a19a30566f1f6</v>
+        <v>N/A</v>
       </c>
       <c r="F69" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G69" t="str">
-        <v>Update Default Values in Suitability Matrix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H69" t="str">
-        <v>Update Default Values in Suitability Matrix</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-19</v>
       </c>
       <c r="B70" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>tin number issue fix and proposal personal detail DM</v>
       </c>
       <c r="C70" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D70">
-        <v>0.62</v>
+        <v>8</v>
       </c>
       <c r="E70" t="str">
-        <v>7bee3eae99c146dd9763677402d811ccdda32634</v>
+        <v>a408a99385e9a653985a56f642fcc28ba2de57e0</v>
       </c>
       <c r="F70" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G70" t="str">
-        <v>Improve Footer Button State Logic</v>
+        <v>tin number issue fix and proposal personal detail DM</v>
       </c>
       <c r="H70" t="str">
-        <v>Improve Footer Button State Logic</v>
+        <v>tin number issue fix and proposal personal detail DM</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B71" t="str">
-        <v>Merge branch 'insure/WE-secureInvest-IGF-bugs' into insure/develop</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C71" t="str">
-        <v>Bug Fix</v>
+        <v>Meeting</v>
       </c>
       <c r="D71">
-        <v>0.62</v>
+        <v>1</v>
       </c>
       <c r="E71" t="str">
-        <v>e99755b1a19ca187ae888f97b657cb3bd62ebbe9</v>
+        <v>N/A</v>
       </c>
       <c r="F71" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G71" t="str">
-        <v>Fix Journey Footer Button Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H71" t="str">
-        <v>Fix Journey Footer Button Logic</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B72" t="str">
-        <v>calculate premium button disable fix</v>
+        <v>single option auto select</v>
       </c>
       <c r="C72" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D72">
-        <v>0.62</v>
+        <v>2</v>
       </c>
       <c r="E72" t="str">
-        <v>5d172e8ac7135918b7c288c0a13dc8ef8d08999c</v>
+        <v>ec9dd5a17c8e072c718bc67e8f05ba8b58e90c53</v>
       </c>
       <c r="F72" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G72" t="str">
-        <v>Fix Premium Button Disabled State</v>
+        <v>single option auto select</v>
       </c>
       <c r="H72" t="str">
-        <v>Fix Premium Button Disabled State</v>
+        <v>single option auto select</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B73" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>dob check uncheck issue fix</v>
       </c>
       <c r="C73" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D73">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="E73" t="str">
-        <v>e7f59082cdabad7472c007815e41b2d2335825b4</v>
+        <v>d168932caf15589c1b9a12a597b27d05a0826231</v>
       </c>
       <c r="F73" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G73" t="str">
-        <v>Implement IGFP Death Cover Component</v>
+        <v>dob check uncheck issue fix</v>
       </c>
       <c r="H73" t="str">
-        <v>Implement IGFP Death Cover Component</v>
+        <v>dob check uncheck issue fix</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B74" t="str">
-        <v>Merge branch 'insure/WE-secureInvest-IGF-bugs' into insure/develop</v>
+        <v>age proof and address proof fix</v>
       </c>
       <c r="C74" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D74">
-        <v>1.23</v>
+        <v>2</v>
       </c>
       <c r="E74" t="str">
-        <v>2847f706999d834011a702f6f3ecc51dece03c77</v>
+        <v>08ac7ff4b44fa4830cd3fd240f46d549e398bf83</v>
       </c>
       <c r="F74" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G74" t="str">
-        <v>Enhance IGFP Death Cover Component</v>
+        <v>age proof and address proof fix</v>
       </c>
       <c r="H74" t="str">
-        <v>Enhance IGFP Death Cover Component</v>
+        <v>age proof and address proof fix</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B75" t="str">
-        <v>death cover factor if igf</v>
+        <v>address type details</v>
       </c>
       <c r="C75" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D75">
-        <v>1.23</v>
+        <v>2</v>
       </c>
       <c r="E75" t="str">
-        <v>239168ecbf49565148eee96ad0a059f9ba259fa4</v>
+        <v>632f1d16ccc018a57846aed8211535da54451d74</v>
       </c>
       <c r="F75" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G75" t="str">
-        <v>Implement Death Cover Feature for IGFP</v>
+        <v>address type details</v>
       </c>
       <c r="H75" t="str">
-        <v>Implement Death Cover Feature for IGFP</v>
+        <v>address type details</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-05-18</v>
+        <v>2026-06-23</v>
       </c>
       <c r="B76" t="str">
-        <v>WE bug of milstone withdrawal option fix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C76" t="str">
-        <v>Bug Fix</v>
+        <v>Meeting</v>
       </c>
       <c r="D76">
-        <v>1.21</v>
+        <v>1</v>
       </c>
       <c r="E76" t="str">
-        <v>1453c7f34e3ddca8b5b61bca423f6e6774fad096</v>
+        <v>N/A</v>
       </c>
       <c r="F76" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G76" t="str">
-        <v>Fix Milestone Withdrawal Option Bug</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H76" t="str">
-        <v>Fix Milestone Withdrawal Option Bug</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-05-19</v>
+        <v>2026-06-23</v>
       </c>
       <c r="B77" t="str">
-        <v>Daily Scrum Call</v>
+        <v>heading driver question</v>
       </c>
       <c r="C77" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>2.67</v>
       </c>
       <c r="E77" t="str">
-        <v>N/A</v>
+        <v>6fb9c4b7629345c302e7ec197ca778d0ef9846cc</v>
       </c>
       <c r="F77" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G77" t="str">
-        <v>Daily Scrum Call</v>
+        <v>heading driver question</v>
       </c>
       <c r="H77" t="str">
-        <v>Daily Scrum Call</v>
+        <v>heading driver question</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-05-19</v>
+        <v>2026-06-23</v>
       </c>
       <c r="B78" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>driver questionar</v>
       </c>
       <c r="C78" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D78">
-        <v>1.23</v>
+        <v>2.67</v>
       </c>
       <c r="E78" t="str">
-        <v>86798a7cdd5e2aae569be6ee3e1f5a7578df68ff</v>
+        <v>2d63fc872425b4c874f97a3dfb2dbafe543b892d</v>
       </c>
       <c r="F78" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G78" t="str">
-        <v>Update Channel Conditions and Add Form Components</v>
+        <v>driver questionar</v>
       </c>
       <c r="H78" t="str">
-        <v>Update Channel Conditions and Add Form Components</v>
+        <v>driver questionar</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-05-19</v>
+        <v>2026-06-23</v>
       </c>
       <c r="B79" t="str">
-        <v>Merge branch 'insure/channel-detailPage' into insure/develop</v>
+        <v>DM-23546</v>
       </c>
       <c r="C79" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D79">
-        <v>1.85</v>
+        <v>2.66</v>
       </c>
       <c r="E79" t="str">
-        <v>a3938cb9fd934342188d0ba5038664b41e1c67fa</v>
+        <v>e2fca5aca7bbd4758ad5ff5bb7331aa403f5c405</v>
       </c>
       <c r="F79" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G79" t="str">
-        <v>Update Channel Details Functionality</v>
+        <v>DM-23546</v>
       </c>
       <c r="H79" t="str">
-        <v>Update Channel Details Functionality</v>
+        <v>DM-23546</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-05-19</v>
+        <v>2026-06-25</v>
       </c>
       <c r="B80" t="str">
-        <v>channel-page integration</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C80" t="str">
-        <v>Feature</v>
+        <v>Meeting</v>
       </c>
       <c r="D80">
-        <v>1.85</v>
+        <v>1</v>
       </c>
       <c r="E80" t="str">
-        <v>8dfa4a91c2e508b0a476b094f90ed0aef53aaafc</v>
+        <v>N/A</v>
       </c>
       <c r="F80" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G80" t="str">
-        <v>Integrate Channel Page with New Features</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H80" t="str">
-        <v>Integrate Channel Page with New Features</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-05-19</v>
+        <v>2026-06-25</v>
       </c>
       <c r="B81" t="str">
-        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/ISNP into insure/develop</v>
+        <v>address and dob always unchecked</v>
       </c>
       <c r="C81" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D81">
-        <v>1.23</v>
+        <v>2</v>
       </c>
       <c r="E81" t="str">
-        <v>b551b4365ba3deb159c3843a4ef5b379aba2629c</v>
+        <v>b4a7f1a6f3ef2cc5efbcc6f5b78dea8804a24a24</v>
       </c>
       <c r="F81" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G81" t="str">
-        <v>Update Financial Analysis Form Defaults</v>
+        <v>address and dob always unchecked</v>
       </c>
       <c r="H81" t="str">
-        <v>Update Financial Analysis Form Defaults</v>
+        <v>address and dob always unchecked</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-05-19</v>
+        <v>2026-06-25</v>
       </c>
       <c r="B82" t="str">
-        <v>alpha wealth started 19 may</v>
+        <v>promise4growthplus DM fixes</v>
       </c>
       <c r="C82" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D82">
-        <v>1.84</v>
+        <v>2</v>
       </c>
       <c r="E82" t="str">
-        <v>0ad33d480ed3c8078e689e14bf7212d5eecf3313</v>
+        <v>b7b3a18ef18378d3c993910abd73ed738440ad3e</v>
       </c>
       <c r="F82" t="str">
-        <v>insure/Alpha-wealth</v>
+        <v>insure/develop</v>
       </c>
       <c r="G82" t="str">
-        <v>Implement Wealth Management Options</v>
+        <v>promise4growthplus DM fixes</v>
       </c>
       <c r="H82" t="str">
-        <v>Implement Wealth Management Options</v>
+        <v>promise4growthplus DM fixes</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-25</v>
       </c>
       <c r="B83" t="str">
-        <v>Daily Scrum Call</v>
+        <v>dock question multiselect</v>
       </c>
       <c r="C83" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E83" t="str">
-        <v>N/A</v>
+        <v>c28f1368399b3c0d8e8f0a3bd21a660001c1ac3f</v>
       </c>
       <c r="F83" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G83" t="str">
-        <v>Daily Scrum Call</v>
+        <v>dock question multiselect</v>
       </c>
       <c r="H83" t="str">
-        <v>Daily Scrum Call</v>
+        <v>dock question multiselect</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-25</v>
       </c>
       <c r="B84" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>LA Medical Details come for form 2 case only</v>
       </c>
       <c r="C84" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D84">
-        <v>0.89</v>
+        <v>2</v>
       </c>
       <c r="E84" t="str">
-        <v>64ed5515347bceba58d483fec986f336ed6e76e4</v>
+        <v>6d9049c8e776a726ab2e2cadf8d2f77ccf2c803d</v>
       </c>
       <c r="F84" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G84" t="str">
-        <v>Update Channel WatchValue to SPECTRUM</v>
+        <v>LA Medical Details come for form 2 case only</v>
       </c>
       <c r="H84" t="str">
-        <v>Update Channel WatchValue to SPECTRUM</v>
+        <v>LA Medical Details come for form 2 case only</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-26</v>
       </c>
       <c r="B85" t="str">
-        <v>Revert "Merge branch 'insure/channel-detailPage' into insure/develop"</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C85" t="str">
-        <v>Bug Fix</v>
+        <v>Meeting</v>
       </c>
       <c r="D85">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E85" t="str">
-        <v>d30332c727d15a7dfb19a6983bfe02d2ee011af8</v>
+        <v>N/A</v>
       </c>
       <c r="F85" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G85" t="str">
-        <v>Update Channel Watch Value for Insurance Journey</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H85" t="str">
-        <v>Update Channel Watch Value for Insurance Journey</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-26</v>
       </c>
       <c r="B86" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>ulip rider plan code</v>
       </c>
       <c r="C86" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D86">
-        <v>1.78</v>
+        <v>2.67</v>
       </c>
       <c r="E86" t="str">
-        <v>d872a95fbc0e03b51efc244d0f4140b831f79d3b</v>
+        <v>84f93450837775e7e63ee19b1ab48edbb7039310</v>
       </c>
       <c r="F86" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G86" t="str">
-        <v>Enhance Fund Allocation Validation Logic</v>
+        <v>ulip rider plan code</v>
       </c>
       <c r="H86" t="str">
-        <v>Enhance Fund Allocation Validation Logic</v>
+        <v>ulip rider plan code</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-26</v>
       </c>
       <c r="B87" t="str">
-        <v>claculate premium button fix</v>
+        <v>dont show harcoded error message on annur</v>
       </c>
       <c r="C87" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D87">
-        <v>1.33</v>
+        <v>2.67</v>
       </c>
       <c r="E87" t="str">
-        <v>6525dc2ab9d0793c593cdb57b644551f436e3c9b</v>
+        <v>e22e159cd06c15111919b9408eb0d1435b301574</v>
       </c>
       <c r="F87" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G87" t="str">
-        <v>Fix Premium Calculation Error Messages</v>
+        <v>dont show harcoded error message on annur</v>
       </c>
       <c r="H87" t="str">
-        <v>Fix Premium Calculation Error Messages</v>
+        <v>dont show harcoded error message on annur</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-26</v>
       </c>
       <c r="B88" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>when no rider directly continue</v>
       </c>
       <c r="C88" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D88">
-        <v>1.33</v>
+        <v>2.66</v>
       </c>
       <c r="E88" t="str">
-        <v>006d95a039ef62d32ccfda84daa96321394a676c</v>
+        <v>c250ba72d7414c93b52250f1a5bbc227aae3d2a0</v>
       </c>
       <c r="F88" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G88" t="str">
-        <v>Enhance Navigation Logic for Payment Process</v>
+        <v>when no rider directly continue</v>
       </c>
       <c r="H88" t="str">
-        <v>Enhance Navigation Logic for Payment Process</v>
+        <v>when no rider directly continue</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-05-20</v>
+        <v>2026-06-29</v>
       </c>
       <c r="B89" t="str">
-        <v>enable calculate premium fix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C89" t="str">
-        <v>Feature</v>
+        <v>Meeting</v>
       </c>
       <c r="D89">
-        <v>1.34</v>
+        <v>1</v>
       </c>
       <c r="E89" t="str">
-        <v>6b8683ccd2598f9b8b5ec8840adf55de365f0544</v>
+        <v>N/A</v>
       </c>
       <c r="F89" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>N/A</v>
       </c>
       <c r="G89" t="str">
-        <v>Enable Premium Calculation Functionality</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H89" t="str">
-        <v>Enable Premium Calculation Functionality</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-05-21</v>
+        <v>2026-06-29</v>
       </c>
       <c r="B90" t="str">
-        <v>Daily Scrum Call</v>
+        <v>open numeric keypad in suatabilyt matrix</v>
       </c>
       <c r="C90" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D90">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E90" t="str">
-        <v>N/A</v>
+        <v>f64f202e90af5d1099e59d83d57f070f934b0d13</v>
       </c>
       <c r="F90" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G90" t="str">
-        <v>Daily Scrum Call</v>
+        <v>open numeric keypad in suatabilyt matrix</v>
       </c>
       <c r="H90" t="str">
-        <v>Daily Scrum Call</v>
+        <v>open numeric keypad in suatabilyt matrix</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-05-21</v>
+        <v>2026-06-29</v>
       </c>
       <c r="B91" t="str">
-        <v>single payment in IGF plan</v>
+        <v>error on generate BI also condiser gernal error</v>
       </c>
       <c r="C91" t="str">
-        <v>Feature</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D91">
-        <v>8</v>
+        <v>1.6</v>
       </c>
       <c r="E91" t="str">
-        <v>1da526a26f0dee753286d3a3b01695d101ac804c</v>
+        <v>48b28334b39accca8f60e61d842d2e08b2e88210</v>
       </c>
       <c r="F91" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G91" t="str">
-        <v>Implement Single Payment Option for IGF Plan</v>
+        <v>error on generate BI also condiser gernal error</v>
       </c>
       <c r="H91" t="str">
-        <v>Implement Single Payment Option for IGF Plan</v>
+        <v>error on generate BI also condiser gernal error</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-05-22</v>
+        <v>2026-06-29</v>
       </c>
       <c r="B92" t="str">
-        <v>Daily Scrum Call</v>
+        <v>promise4growthplus ppt value isssue fix</v>
       </c>
       <c r="C92" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D92">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="E92" t="str">
-        <v>N/A</v>
+        <v>8d7da8462d1558b346eafda60080e9e917abdc18</v>
       </c>
       <c r="F92" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G92" t="str">
-        <v>Daily Scrum Call</v>
+        <v>promise4growthplus ppt value isssue fix</v>
       </c>
       <c r="H92" t="str">
-        <v>Daily Scrum Call</v>
+        <v>promise4growthplus ppt value isssue fix</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-05-22</v>
+        <v>2026-06-29</v>
       </c>
       <c r="B93" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
+        <v>height,weight decial logic same as ISNP</v>
       </c>
       <c r="C93" t="str">
-        <v>Refactor</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D93">
-        <v>1.78</v>
+        <v>1.6</v>
       </c>
       <c r="E93" t="str">
-        <v>09a96d4abd371fb5281df6892169dc38896a67e6</v>
+        <v>4dfa9dd3d803e4ec3ea56f32a63850c2a4bcbbd7</v>
       </c>
       <c r="F93" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G93" t="str">
-        <v>Refactor Investment Plan Form Fields</v>
+        <v>height,weight decial logic same as ISNP</v>
       </c>
       <c r="H93" t="str">
-        <v>Refactor Investment Plan Form Fields</v>
+        <v>height,weight decial logic same as ISNP</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2026-05-22</v>
+        <v>2026-06-29</v>
       </c>
       <c r="B94" t="str">
-        <v>Revert "fix wealth edge bugs"</v>
+        <v>training api byass temp</v>
       </c>
       <c r="C94" t="str">
-        <v>Bug Fix</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D94">
-        <v>0.89</v>
+        <v>1.6</v>
       </c>
       <c r="E94" t="str">
-        <v>0dc2e1bf1308350297573931fc237a2922f45324</v>
+        <v>9a8e40da79daed6e65fd0e6ae77f596a4852e663</v>
       </c>
       <c r="F94" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G94" t="str">
-        <v>Revert PDF Library Updates</v>
+        <v>training api byass temp</v>
       </c>
       <c r="H94" t="str">
-        <v>Revert PDF Library Updates</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <v>2026-05-22</v>
-      </c>
-      <c r="B95" t="str">
-        <v>fix wealth edge bugs</v>
-      </c>
-      <c r="C95" t="str">
-        <v>Bug Fix</v>
-      </c>
-      <c r="D95">
-        <v>1.78</v>
-      </c>
-      <c r="E95" t="str">
-        <v>194a2a10d5648c12f59eb9170d0d12837eb04801</v>
-      </c>
-      <c r="F95" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G95" t="str">
-        <v>Fix Bugs in Wealth Edge Application</v>
-      </c>
-      <c r="H95" t="str">
-        <v>Fix Bugs in Wealth Edge Application</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="str">
-        <v>2026-05-22</v>
-      </c>
-      <c r="B96" t="str">
-        <v>wealth Edge fix</v>
-      </c>
-      <c r="C96" t="str">
-        <v>Refactor</v>
-      </c>
-      <c r="D96">
-        <v>1.78</v>
-      </c>
-      <c r="E96" t="str">
-        <v>16e6f667d869ca1738a2918042769f6883d4328e</v>
-      </c>
-      <c r="F96" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G96" t="str">
-        <v>Refactor Wealth Edge Sum Assured Validation</v>
-      </c>
-      <c r="H96" t="str">
-        <v>Refactor Wealth Edge Sum Assured Validation</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>2026-05-22</v>
-      </c>
-      <c r="B97" t="str">
-        <v>Merge branch 'insure/develop' of https://github.com/lumiqai/ISNP into insure/develop</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="D97">
-        <v>1.77</v>
-      </c>
-      <c r="E97" t="str">
-        <v>f297407b36b06b2fd5d27ce6d9df6415982aa0c4</v>
-      </c>
-      <c r="F97" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G97" t="str">
-        <v>Enhance Insurance Proposal Interface</v>
-      </c>
-      <c r="H97" t="str">
-        <v>Enhance Insurance Proposal Interface</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>2026-05-26</v>
-      </c>
-      <c r="B98" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-      <c r="C98" t="str">
-        <v>Meeting</v>
-      </c>
-      <c r="D98">
-        <v>1</v>
-      </c>
-      <c r="E98" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="F98" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="G98" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-      <c r="H98" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>2026-05-26</v>
-      </c>
-      <c r="B99" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
-      </c>
-      <c r="C99" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="D99">
-        <v>4.57</v>
-      </c>
-      <c r="E99" t="str">
-        <v>cdb73e50a9b95bd1f3febf4a47ee136cc0eb7ca7</v>
-      </c>
-      <c r="F99" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G99" t="str">
-        <v>Enhance Nominee Button Functionality</v>
-      </c>
-      <c r="H99" t="str">
-        <v>Enhance Nominee Button Functionality</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>2026-05-26</v>
-      </c>
-      <c r="B100" t="str">
-        <v>DM-22967 add nominee disable after 100%</v>
-      </c>
-      <c r="C100" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="D100">
-        <v>3.43</v>
-      </c>
-      <c r="E100" t="str">
-        <v>ee50b94669ab68b4c4fa5ed581ed46c49058db40</v>
-      </c>
-      <c r="F100" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G100" t="str">
-        <v>Implement Nominee Addition Logic</v>
-      </c>
-      <c r="H100" t="str">
-        <v>Implement Nominee Addition Logic</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>2026-05-27</v>
-      </c>
-      <c r="B101" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-      <c r="C101" t="str">
-        <v>Meeting</v>
-      </c>
-      <c r="D101">
-        <v>1</v>
-      </c>
-      <c r="E101" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="F101" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="G101" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-      <c r="H101" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="str">
-        <v>2026-05-27</v>
-      </c>
-      <c r="B102" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
-      </c>
-      <c r="C102" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="D102">
-        <v>4</v>
-      </c>
-      <c r="E102" t="str">
-        <v>1d6af1b12b3797600fa64b4d7e696e97e2cedaea</v>
-      </c>
-      <c r="F102" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G102" t="str">
-        <v>Enhance IGFP Premium Protection Cover Logic</v>
-      </c>
-      <c r="H102" t="str">
-        <v>Enhance IGFP Premium Protection Cover Logic</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="str">
-        <v>2026-05-27</v>
-      </c>
-      <c r="B103" t="str">
-        <v>payor ppc feature igf plan</v>
-      </c>
-      <c r="C103" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="D103">
-        <v>4</v>
-      </c>
-      <c r="E103" t="str">
-        <v>f9af1886590768acf59cc5bb6392e582f0cd9ae5</v>
-      </c>
-      <c r="F103" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G103" t="str">
-        <v>Implement Premium Protection Cover Feature</v>
-      </c>
-      <c r="H103" t="str">
-        <v>Implement Premium Protection Cover Feature</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="str">
-        <v>2026-05-29</v>
-      </c>
-      <c r="B104" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-      <c r="C104" t="str">
-        <v>Meeting</v>
-      </c>
-      <c r="D104">
-        <v>1</v>
-      </c>
-      <c r="E104" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="F104" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="G104" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-      <c r="H104" t="str">
-        <v>Daily Scrum Call</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="str">
-        <v>2026-05-29</v>
-      </c>
-      <c r="B105" t="str">
-        <v>Merge branch 'insure/develop' into infinityInsure2.0/uat</v>
-      </c>
-      <c r="C105" t="str">
-        <v>Feature</v>
-      </c>
-      <c r="D105">
-        <v>4</v>
-      </c>
-      <c r="E105" t="str">
-        <v>e48236e65795ac0b0f8b776654f4f90626dc4f49</v>
-      </c>
-      <c r="F105" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G105" t="str">
-        <v>Implement Agent Relationship Logic in Payment Flow</v>
-      </c>
-      <c r="H105" t="str">
-        <v>Implement Agent Relationship Logic in Payment Flow</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="str">
-        <v>2026-05-29</v>
-      </c>
-      <c r="B106" t="str">
-        <v>condtional otp api fix</v>
-      </c>
-      <c r="C106" t="str">
-        <v>Bug Fix</v>
-      </c>
-      <c r="D106">
-        <v>4</v>
-      </c>
-      <c r="E106" t="str">
-        <v>d7a96eea0b41afe48263a5a08e47d4338afdaf15</v>
-      </c>
-      <c r="F106" t="str">
-        <v>infinityInsure2.0/uat</v>
-      </c>
-      <c r="G106" t="str">
-        <v>Fix OTP API Conditional Logic</v>
-      </c>
-      <c r="H106" t="str">
-        <v>Fix OTP API Conditional Logic</v>
+        <v>training api byass temp</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H106"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H94"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update frontend to support multiple repositories and implement direct APU sheet generation for Redmine logging.
</commit_message>
<xml_diff>
--- a/redmine-logger/backend/user_data/lumiqshubh23/git_commits.xlsx
+++ b/redmine-logger/backend/user_data/lumiqshubh23/git_commits.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="DD-MMM-YYYY"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -397,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H126"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -462,7 +463,7 @@
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D3">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="E3" t="str">
         <v>5033a821c6e25b95378953140ed14edca12d0e84</v>
@@ -488,7 +489,7 @@
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D4">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="E4" t="str">
         <v>7772684e682945f39c9cd52d75cb5bdb0c27e994</v>
@@ -514,7 +515,7 @@
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D5">
-        <v>2.66</v>
+        <v>2</v>
       </c>
       <c r="E5" t="str">
         <v>d1b7e2f9d0fc330e4ec7fbf4b0baf95ef0b0f544</v>
@@ -531,28 +532,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-06-02</v>
+        <v>2026-06-01</v>
       </c>
       <c r="B6" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-22984 deathcover factor in igf</v>
       </c>
       <c r="C6" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="str">
-        <v>N/A</v>
+        <v>4da85214ae597eb1e2f8374528e43ce57fb426da</v>
       </c>
       <c r="F6" t="str">
-        <v>N/A</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G6" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-22984 deathcover factor in igf</v>
       </c>
       <c r="H6" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-22984 deathcover factor in igf</v>
       </c>
     </row>
     <row r="7">
@@ -560,25 +561,25 @@
         <v>2026-06-02</v>
       </c>
       <c r="B7" t="str">
-        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C7" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D7">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>09c6c080804f72a8df6c44653f478851330fccd8</v>
+        <v>N/A</v>
       </c>
       <c r="F7" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G7" t="str">
-        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H7" t="str">
-        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="8">
@@ -586,25 +587,25 @@
         <v>2026-06-02</v>
       </c>
       <c r="B8" t="str">
-        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
+        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
       </c>
       <c r="C8" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D8">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>15bd27fe6965ad8aa560d25a8a9f8c20cb5f1dd4</v>
+        <v>09c6c080804f72a8df6c44653f478851330fccd8</v>
       </c>
       <c r="F8" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G8" t="str">
-        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
+        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
       </c>
       <c r="H8" t="str">
-        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
+        <v>DM-23087 The “Are you opting for Staff Discount?” option should be placed after the “Annual Income” field.</v>
       </c>
     </row>
     <row r="9">
@@ -612,25 +613,25 @@
         <v>2026-06-02</v>
       </c>
       <c r="B9" t="str">
-        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
+        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
       </c>
       <c r="C9" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D9">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>eb7cf33323d4a62471b0bbea27611f71d129673d</v>
+        <v>15bd27fe6965ad8aa560d25a8a9f8c20cb5f1dd4</v>
       </c>
       <c r="F9" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G9" t="str">
-        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
+        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
       </c>
       <c r="H9" t="str">
-        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
+        <v>DM-23089 "Are you opting for Staff Discount?"option is currently displayed in the Life Assured (LA) Details section</v>
       </c>
     </row>
     <row r="10">
@@ -638,25 +639,25 @@
         <v>2026-06-02</v>
       </c>
       <c r="B10" t="str">
-        <v>DM-23070 Pincode api run after clicking outside the field</v>
+        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
       </c>
       <c r="C10" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D10">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>45239ff3a1193cb91d9b366fda2e615d55aaf5ed</v>
+        <v>eb7cf33323d4a62471b0bbea27611f71d129673d</v>
       </c>
       <c r="F10" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G10" t="str">
-        <v>DM-23070 Pincode api run after clicking outside the field</v>
+        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
       </c>
       <c r="H10" t="str">
-        <v>DM-23070 Pincode api run after clicking outside the field</v>
+        <v>DM-22975 || Validation need to be implement for Illiterate Education</v>
       </c>
     </row>
     <row r="11">
@@ -664,25 +665,25 @@
         <v>2026-06-02</v>
       </c>
       <c r="B11" t="str">
-        <v>secure Invest afr fix</v>
+        <v>DM-23070 Pincode api run after clicking outside the field</v>
       </c>
       <c r="C11" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D11">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E11" t="str">
-        <v>38d50b8f7fac49f9b16d29c8582958bbb40ae9ff</v>
+        <v>45239ff3a1193cb91d9b366fda2e615d55aaf5ed</v>
       </c>
       <c r="F11" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G11" t="str">
-        <v>secure Invest afr fix</v>
+        <v>DM-23070 Pincode api run after clicking outside the field</v>
       </c>
       <c r="H11" t="str">
-        <v>secure Invest afr fix</v>
+        <v>DM-23070 Pincode api run after clicking outside the field</v>
       </c>
     </row>
     <row r="12">
@@ -696,10 +697,10 @@
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D12">
-        <v>1.35</v>
+        <v>1</v>
       </c>
       <c r="E12" t="str">
-        <v>5e4a4a77c57a009e00e9661f54a8f2b620d3e266</v>
+        <v>38d50b8f7fac49f9b16d29c8582958bbb40ae9ff</v>
       </c>
       <c r="F12" t="str">
         <v>insure/develop</v>
@@ -713,36 +714,36 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-06-03</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B13" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secure Invest afr fix</v>
       </c>
       <c r="C13" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" t="str">
-        <v>N/A</v>
+        <v>5e4a4a77c57a009e00e9661f54a8f2b620d3e266</v>
       </c>
       <c r="F13" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G13" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secure Invest afr fix</v>
       </c>
       <c r="H13" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secure Invest afr fix</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-06-03</v>
+        <v>2026-06-02</v>
       </c>
       <c r="B14" t="str">
-        <v>Revert "alternative number added"</v>
+        <v>AFR secureInvest fix</v>
       </c>
       <c r="C14" t="str">
         <v>Development &amp; Configuration</v>
@@ -751,16 +752,16 @@
         <v>2</v>
       </c>
       <c r="E14" t="str">
-        <v>60606c0a103f76c72422f3155668650136edcd40</v>
+        <v>739b615da1d9543e4789cb3344123091ec373359</v>
       </c>
       <c r="F14" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G14" t="str">
-        <v>Revert "alternative number added"</v>
+        <v>AFR secureInvest fix</v>
       </c>
       <c r="H14" t="str">
-        <v>Revert "alternative number added"</v>
+        <v>AFR secureInvest fix</v>
       </c>
     </row>
     <row r="15">
@@ -768,25 +769,25 @@
         <v>2026-06-03</v>
       </c>
       <c r="B15" t="str">
-        <v>alternative number added</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C15" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" t="str">
-        <v>370237486317451707c49b64a237b56148ad9bc7</v>
+        <v>N/A</v>
       </c>
       <c r="F15" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G15" t="str">
-        <v>alternative number added</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H15" t="str">
-        <v>alternative number added</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="16">
@@ -794,25 +795,25 @@
         <v>2026-06-03</v>
       </c>
       <c r="B16" t="str">
-        <v>rop error msg fix</v>
+        <v>Revert "alternative number added"</v>
       </c>
       <c r="C16" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="str">
-        <v>b37bc9ee06f2575abaa1113396367f1ac801bdff</v>
+        <v>60606c0a103f76c72422f3155668650136edcd40</v>
       </c>
       <c r="F16" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G16" t="str">
-        <v>rop error msg fix</v>
+        <v>Revert "alternative number added"</v>
       </c>
       <c r="H16" t="str">
-        <v>rop error msg fix</v>
+        <v>Revert "alternative number added"</v>
       </c>
     </row>
     <row r="17">
@@ -820,181 +821,181 @@
         <v>2026-06-03</v>
       </c>
       <c r="B17" t="str">
-        <v>wealth edge fund issue fix</v>
+        <v>alternative number added</v>
       </c>
       <c r="C17" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="str">
-        <v>a3c9496d6ae1e5d5bed1bff81002ff7360c4d36a</v>
+        <v>370237486317451707c49b64a237b56148ad9bc7</v>
       </c>
       <c r="F17" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G17" t="str">
-        <v>wealth edge fund issue fix</v>
+        <v>alternative number added</v>
       </c>
       <c r="H17" t="str">
-        <v>wealth edge fund issue fix</v>
+        <v>alternative number added</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B18" t="str">
-        <v>Daily Scrum Call</v>
+        <v>rop error msg fix</v>
       </c>
       <c r="C18" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v>N/A</v>
+        <v>b37bc9ee06f2575abaa1113396367f1ac801bdff</v>
       </c>
       <c r="F18" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G18" t="str">
-        <v>Daily Scrum Call</v>
+        <v>rop error msg fix</v>
       </c>
       <c r="H18" t="str">
-        <v>Daily Scrum Call</v>
+        <v>rop error msg fix</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B19" t="str">
-        <v>spelling mistake fix</v>
+        <v>wealth edge fund issue fix</v>
       </c>
       <c r="C19" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D19">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E19" t="str">
-        <v>4a829a71dfd645d746a114dcaeabd3646dfd11f4</v>
+        <v>a3c9496d6ae1e5d5bed1bff81002ff7360c4d36a</v>
       </c>
       <c r="F19" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G19" t="str">
-        <v>spelling mistake fix</v>
+        <v>wealth edge fund issue fix</v>
       </c>
       <c r="H19" t="str">
-        <v>spelling mistake fix</v>
+        <v>wealth edge fund issue fix</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B20" t="str">
-        <v>mariner field issue</v>
+        <v>Revert "alternative number issue fix"</v>
       </c>
       <c r="C20" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D20">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E20" t="str">
-        <v>6f8e7ceed8731e893cf5fc9d2577123d8cd996f3</v>
+        <v>8dd15cad942ac9c5b1b38cb21d1771c9a1174106</v>
       </c>
       <c r="F20" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G20" t="str">
-        <v>mariner field issue</v>
+        <v>Revert "alternative number issue fix"</v>
       </c>
       <c r="H20" t="str">
-        <v>mariner field issue</v>
+        <v>Revert "alternative number issue fix"</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B21" t="str">
-        <v>wealth edge continue issue fix</v>
+        <v>Revert "alternative number issue fix"</v>
       </c>
       <c r="C21" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D21">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E21" t="str">
-        <v>76bc99847e8c16318d11785e10b6e8abc52001c1</v>
+        <v>0a55e9ebf9206acc4b9644f3bb288f73e8b9e9ab</v>
       </c>
       <c r="F21" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G21" t="str">
-        <v>wealth edge continue issue fix</v>
+        <v>Revert "alternative number issue fix"</v>
       </c>
       <c r="H21" t="str">
-        <v>wealth edge continue issue fix</v>
+        <v>Revert "alternative number issue fix"</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B22" t="str">
-        <v>bi pdf through sms</v>
+        <v>alternative number issue fix</v>
       </c>
       <c r="C22" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D22">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E22" t="str">
-        <v>af1fabf41c1901c58a4535fe6c49933536afed1c</v>
+        <v>4d9ff2bbc2940e10af61c44bbdf114ec1da39cce</v>
       </c>
       <c r="F22" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G22" t="str">
-        <v>bi pdf through sms</v>
+        <v>alternative number issue fix</v>
       </c>
       <c r="H22" t="str">
-        <v>bi pdf through sms</v>
+        <v>alternative number issue fix</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-03</v>
       </c>
       <c r="B23" t="str">
-        <v>DM-23175</v>
+        <v>wealth edge fund issue fix</v>
       </c>
       <c r="C23" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D23">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E23" t="str">
-        <v>0dd43a17d6c491ce1212b63b140285018b28922e</v>
+        <v>b056e72bb1427b69544bc2672d0fef06b2d8aa00</v>
       </c>
       <c r="F23" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G23" t="str">
-        <v>DM-23175</v>
+        <v>wealth edge fund issue fix</v>
       </c>
       <c r="H23" t="str">
-        <v>DM-23175</v>
+        <v>wealth edge fund issue fix</v>
       </c>
     </row>
     <row r="24">
@@ -1002,25 +1003,25 @@
         <v>2026-06-04</v>
       </c>
       <c r="B24" t="str">
-        <v>DM-22975 illitrate mapping</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C24" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D24">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E24" t="str">
-        <v>cbaaa9fedfb48e753e7ee7c11737ea9887fb225f</v>
+        <v>N/A</v>
       </c>
       <c r="F24" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G24" t="str">
-        <v>DM-22975 illitrate mapping</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H24" t="str">
-        <v>DM-22975 illitrate mapping</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="25">
@@ -1028,264 +1029,264 @@
         <v>2026-06-04</v>
       </c>
       <c r="B25" t="str">
-        <v>address flow chnage</v>
+        <v>spelling mistake fix</v>
       </c>
       <c r="C25" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D25">
-        <v>1.16</v>
+        <v>1</v>
       </c>
       <c r="E25" t="str">
-        <v>bbca155bf05e640939b18486d9a0e0b20f7cf62e</v>
+        <v>4a829a71dfd645d746a114dcaeabd3646dfd11f4</v>
       </c>
       <c r="F25" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G25" t="str">
-        <v>address flow chnage</v>
+        <v>spelling mistake fix</v>
       </c>
       <c r="H25" t="str">
-        <v>address flow chnage</v>
+        <v>spelling mistake fix</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B26" t="str">
-        <v>Daily Scrum Call</v>
+        <v>mariner field issue</v>
       </c>
       <c r="C26" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D26">
         <v>1</v>
       </c>
       <c r="E26" t="str">
-        <v>N/A</v>
+        <v>6f8e7ceed8731e893cf5fc9d2577123d8cd996f3</v>
       </c>
       <c r="F26" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G26" t="str">
-        <v>Daily Scrum Call</v>
+        <v>mariner field issue</v>
       </c>
       <c r="H26" t="str">
-        <v>Daily Scrum Call</v>
+        <v>mariner field issue</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B27" t="str">
-        <v>secure invest sto fund logic</v>
+        <v>wealth edge continue issue fix</v>
       </c>
       <c r="C27" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D27">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E27" t="str">
-        <v>0f8491441ef27c57ea6a99411132fb25e32eda21</v>
+        <v>76bc99847e8c16318d11785e10b6e8abc52001c1</v>
       </c>
       <c r="F27" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G27" t="str">
-        <v>secure invest sto fund logic</v>
+        <v>wealth edge continue issue fix</v>
       </c>
       <c r="H27" t="str">
-        <v>secure invest sto fund logic</v>
+        <v>wealth edge continue issue fix</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B28" t="str">
-        <v>Revert "DM-23121 if single option then autoSelect"</v>
+        <v>bi pdf through sms</v>
       </c>
       <c r="C28" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D28">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E28" t="str">
-        <v>298c2849370ac0d64d6c362b14e9ebdb63501646</v>
+        <v>af1fabf41c1901c58a4535fe6c49933536afed1c</v>
       </c>
       <c r="F28" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G28" t="str">
-        <v>Revert "DM-23121 if single option then autoSelect"</v>
+        <v>bi pdf through sms</v>
       </c>
       <c r="H28" t="str">
-        <v>Revert "DM-23121 if single option then autoSelect"</v>
+        <v>bi pdf through sms</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B29" t="str">
-        <v>aadhar masked when 12 diigit</v>
+        <v>DM-23175</v>
       </c>
       <c r="C29" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D29">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E29" t="str">
-        <v>42e680234bb7454719e3e454aa541d9cda441ab4</v>
+        <v>0dd43a17d6c491ce1212b63b140285018b28922e</v>
       </c>
       <c r="F29" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G29" t="str">
-        <v>aadhar masked when 12 diigit</v>
+        <v>DM-23175</v>
       </c>
       <c r="H29" t="str">
-        <v>aadhar masked when 12 diigit</v>
+        <v>DM-23175</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B30" t="str">
-        <v>DM-23121 if single option then autoSelect</v>
+        <v>DM-22975 illitrate mapping</v>
       </c>
       <c r="C30" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D30">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E30" t="str">
-        <v>093f9840d78111faaa0b8ba1bc26b576dd7b76ac</v>
+        <v>cbaaa9fedfb48e753e7ee7c11737ea9887fb225f</v>
       </c>
       <c r="F30" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G30" t="str">
-        <v>DM-23121 if single option then autoSelect</v>
+        <v>DM-22975 illitrate mapping</v>
       </c>
       <c r="H30" t="str">
-        <v>DM-23121 if single option then autoSelect</v>
+        <v>DM-22975 illitrate mapping</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-06-05</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B31" t="str">
-        <v>DM-23121 if single option then autoSelect</v>
+        <v>address flow chnage</v>
       </c>
       <c r="C31" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D31">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E31" t="str">
-        <v>696502680c74817d742c55d8828822a6980de037</v>
+        <v>bbca155bf05e640939b18486d9a0e0b20f7cf62e</v>
       </c>
       <c r="F31" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G31" t="str">
-        <v>DM-23121 if single option then autoSelect</v>
+        <v>address flow chnage</v>
       </c>
       <c r="H31" t="str">
-        <v>DM-23121 if single option then autoSelect</v>
+        <v>address flow chnage</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-06-09</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B32" t="str">
-        <v>Daily Scrum Call</v>
+        <v>annur address fallback</v>
       </c>
       <c r="C32" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D32">
         <v>1</v>
       </c>
       <c r="E32" t="str">
-        <v>N/A</v>
+        <v>678fc16bb8739ee547ad73d3f0bd1f5c54e505b9</v>
       </c>
       <c r="F32" t="str">
-        <v>N/A</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G32" t="str">
-        <v>Daily Scrum Call</v>
+        <v>annur address fallback</v>
       </c>
       <c r="H32" t="str">
-        <v>Daily Scrum Call</v>
+        <v>annur address fallback</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-06-09</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B33" t="str">
-        <v>secure invest not fund auto select</v>
+        <v>bi pdf send by sms</v>
       </c>
       <c r="C33" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D33">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E33" t="str">
-        <v>39fd1833bc250a89717977e1e3283d43130b3287</v>
+        <v>f7c649e597a497bbe9ff905d9a892829c304b7dd</v>
       </c>
       <c r="F33" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G33" t="str">
-        <v>secure invest not fund auto select</v>
+        <v>bi pdf send by sms</v>
       </c>
       <c r="H33" t="str">
-        <v>secure invest not fund auto select</v>
+        <v>bi pdf send by sms</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-06-09</v>
+        <v>2026-06-04</v>
       </c>
       <c r="B34" t="str">
-        <v>annur wealth edge issue fix</v>
+        <v>address flow change</v>
       </c>
       <c r="C34" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D34">
-        <v>4</v>
+        <v>-1</v>
       </c>
       <c r="E34" t="str">
-        <v>50f6c88d2c7fbab5c57efaa5723a34b71f4386a0</v>
+        <v>21892dc6f20330ce73fb39e694fcf32a02f82fb2</v>
       </c>
       <c r="F34" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G34" t="str">
-        <v>annur wealth edge issue fix</v>
+        <v>address flow change</v>
       </c>
       <c r="H34" t="str">
-        <v>annur wealth edge issue fix</v>
+        <v>address flow change</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-06-10</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B35" t="str">
         <v>Daily Scrum Call</v>
@@ -1311,241 +1312,241 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-06-10</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B36" t="str">
-        <v>secureInvest liquide fund issue fix</v>
+        <v>secure invest sto fund logic</v>
       </c>
       <c r="C36" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D36">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E36" t="str">
-        <v>db04074e51693acf46994b47b89ae6221301b597</v>
+        <v>0f8491441ef27c57ea6a99411132fb25e32eda21</v>
       </c>
       <c r="F36" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G36" t="str">
-        <v>secureInvest liquide fund issue fix</v>
+        <v>secure invest sto fund logic</v>
       </c>
       <c r="H36" t="str">
-        <v>secureInvest liquide fund issue fix</v>
+        <v>secure invest sto fund logic</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-06-10</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B37" t="str">
-        <v>secureInvest whole life option</v>
+        <v>Revert "DM-23121 if single option then autoSelect"</v>
       </c>
       <c r="C37" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D37">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E37" t="str">
-        <v>01fb61970864ac23e69baf11116af08bba99c552</v>
+        <v>298c2849370ac0d64d6c362b14e9ebdb63501646</v>
       </c>
       <c r="F37" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G37" t="str">
-        <v>secureInvest whole life option</v>
+        <v>Revert "DM-23121 if single option then autoSelect"</v>
       </c>
       <c r="H37" t="str">
-        <v>secureInvest whole life option</v>
+        <v>Revert "DM-23121 if single option then autoSelect"</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B38" t="str">
-        <v>Daily Scrum Call</v>
+        <v>aadhar masked when 12 diigit</v>
       </c>
       <c r="C38" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D38">
         <v>1</v>
       </c>
       <c r="E38" t="str">
-        <v>N/A</v>
+        <v>42e680234bb7454719e3e454aa541d9cda441ab4</v>
       </c>
       <c r="F38" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G38" t="str">
-        <v>Daily Scrum Call</v>
+        <v>aadhar masked when 12 diigit</v>
       </c>
       <c r="H38" t="str">
-        <v>Daily Scrum Call</v>
+        <v>aadhar masked when 12 diigit</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B39" t="str">
-        <v>uncheck dob feature</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="C39" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D39">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E39" t="str">
-        <v>ead293f3b06815288e7967a7bb7e52107e7f6c94</v>
+        <v>093f9840d78111faaa0b8ba1bc26b576dd7b76ac</v>
       </c>
       <c r="F39" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G39" t="str">
-        <v>uncheck dob feature</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="H39" t="str">
-        <v>uncheck dob feature</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B40" t="str">
-        <v>adress flow change by enhancement</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="C40" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D40">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E40" t="str">
-        <v>3097285a98b6d6a00da498f480f76072c6e1c592</v>
+        <v>696502680c74817d742c55d8828822a6980de037</v>
       </c>
       <c r="F40" t="str">
-        <v>insure/develop</v>
+        <v>infinityInsure2.0/uat</v>
       </c>
       <c r="G40" t="str">
-        <v>adress flow change by enhancement</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
       <c r="H40" t="str">
-        <v>adress flow change by enhancement</v>
+        <v>DM-23121 if single option then autoSelect</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-05</v>
       </c>
       <c r="B41" t="str">
-        <v>address enhanacement</v>
+        <v>Revert "Merge branch 'uat-common-backend-1' into insure/develop"</v>
       </c>
       <c r="C41" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D41">
-        <v>1.33</v>
+        <v>3</v>
       </c>
       <c r="E41" t="str">
-        <v>1df15fe16d18561d9ae557d4af7f483a2d1939df</v>
+        <v>75654a7b2f75608ca72a4aabd3173ab2bc0b8220</v>
       </c>
       <c r="F41" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G41" t="str">
-        <v>address enhanacement</v>
+        <v>Revert "Merge branch 'uat-common-backend-1' into insure/develop"</v>
       </c>
       <c r="H41" t="str">
-        <v>address enhanacement</v>
+        <v>Revert "Merge branch 'uat-common-backend-1' into insure/develop"</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-08</v>
       </c>
       <c r="B42" t="str">
-        <v>annur navigate to next even if api fail</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C42" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D42">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E42" t="str">
-        <v>c7f0f41075db3410129cceeaf5f971b6c742e667</v>
+        <v>N/A</v>
       </c>
       <c r="F42" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G42" t="str">
-        <v>annur navigate to next even if api fail</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H42" t="str">
-        <v>annur navigate to next even if api fail</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-08</v>
       </c>
       <c r="B43" t="str">
-        <v>add speical character validation on address</v>
+        <v>address issue fix</v>
       </c>
       <c r="C43" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D43">
-        <v>1.33</v>
+        <v>4</v>
       </c>
       <c r="E43" t="str">
-        <v>a385b36d4af4fbaa692a2bb9c9b9d071bdf973d7</v>
+        <v>7637c5f2c4be9ed9ed8935f70d6dc7b30440f6b8</v>
       </c>
       <c r="F43" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G43" t="str">
-        <v>add speical character validation on address</v>
+        <v>address issue fix</v>
       </c>
       <c r="H43" t="str">
-        <v>add speical character validation on address</v>
+        <v>address issue fix</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-06-11</v>
+        <v>2026-06-08</v>
       </c>
       <c r="B44" t="str">
-        <v>wealth edge issue fix</v>
+        <v>unified launch fix</v>
       </c>
       <c r="C44" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D44">
-        <v>1.35</v>
+        <v>4</v>
       </c>
       <c r="E44" t="str">
-        <v>ac9e7046f9f21089761a6d96c097f94bb0ed7165</v>
+        <v>91050bad32cff7f947f03d8dbb655eefeb526da6</v>
       </c>
       <c r="F44" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G44" t="str">
-        <v>wealth edge issue fix</v>
+        <v>unified launch fix</v>
       </c>
       <c r="H44" t="str">
-        <v>wealth edge issue fix</v>
+        <v>unified launch fix</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B45" t="str">
         <v>Daily Scrum Call</v>
@@ -1571,891 +1572,891 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B46" t="str">
-        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
+        <v>secure invest not fund auto select</v>
       </c>
       <c r="C46" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D46">
-        <v>1.14</v>
+        <v>2</v>
       </c>
       <c r="E46" t="str">
-        <v>4f07e17fae2fa8cb32e3bf179b06b7e20fe8942f</v>
+        <v>39fd1833bc250a89717977e1e3283d43130b3287</v>
       </c>
       <c r="F46" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G46" t="str">
-        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
+        <v>secure invest not fund auto select</v>
       </c>
       <c r="H46" t="str">
-        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
+        <v>secure invest not fund auto select</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B47" t="str">
-        <v>pan number must be 10</v>
+        <v>annur wealth edge issue fix</v>
       </c>
       <c r="C47" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D47">
-        <v>1.14</v>
+        <v>2</v>
       </c>
       <c r="E47" t="str">
-        <v>6cf0060bb8f1341fd076662f36f21ea3ff1bf2e5</v>
+        <v>50f6c88d2c7fbab5c57efaa5723a34b71f4386a0</v>
       </c>
       <c r="F47" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G47" t="str">
-        <v>pan number must be 10</v>
+        <v>annur wealth edge issue fix</v>
       </c>
       <c r="H47" t="str">
-        <v>pan number must be 10</v>
+        <v>annur wealth edge issue fix</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-09</v>
       </c>
       <c r="B48" t="str">
-        <v>Relationship with PEP other field add</v>
+        <v>annur wealth edge issue fix</v>
       </c>
       <c r="C48" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D48">
-        <v>1.14</v>
+        <v>4</v>
       </c>
       <c r="E48" t="str">
-        <v>37de77bf0a1c9579237aa77cced98d5f64dfd18c</v>
+        <v>fb98a858a1d9171ad1034e58e522088a2de06040</v>
       </c>
       <c r="F48" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G48" t="str">
-        <v>Relationship with PEP other field add</v>
+        <v>annur wealth edge issue fix</v>
       </c>
       <c r="H48" t="str">
-        <v>Relationship with PEP other field add</v>
+        <v>annur wealth edge issue fix</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B49" t="str">
-        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C49" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D49">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="E49" t="str">
-        <v>54688bbceecfe9edf3baff9717ace090b07f228f</v>
+        <v>N/A</v>
       </c>
       <c r="F49" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G49" t="str">
-        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H49" t="str">
-        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B50" t="str">
-        <v>PO personal Health details should not come for form 2 cases</v>
+        <v>secureInvest liquide fund issue fix</v>
       </c>
       <c r="C50" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D50">
-        <v>1.14</v>
+        <v>2</v>
       </c>
       <c r="E50" t="str">
-        <v>d9b9549bf78158a844a9ce66cea71510c9ba251b</v>
+        <v>db04074e51693acf46994b47b89ae6221301b597</v>
       </c>
       <c r="F50" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G50" t="str">
-        <v>PO personal Health details should not come for form 2 cases</v>
+        <v>secureInvest liquide fund issue fix</v>
       </c>
       <c r="H50" t="str">
-        <v>PO personal Health details should not come for form 2 cases</v>
+        <v>secureInvest liquide fund issue fix</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B51" t="str">
-        <v>for 2 case questionior handle</v>
+        <v>secureInvest whole life option</v>
       </c>
       <c r="C51" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D51">
-        <v>1.14</v>
+        <v>2</v>
       </c>
       <c r="E51" t="str">
-        <v>09fd7f027227956b052b1b960c1097944cb1a60f</v>
+        <v>01fb61970864ac23e69baf11116af08bba99c552</v>
       </c>
       <c r="F51" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G51" t="str">
-        <v>for 2 case questionior handle</v>
+        <v>secureInvest whole life option</v>
       </c>
       <c r="H51" t="str">
-        <v>for 2 case questionior handle</v>
+        <v>secureInvest whole life option</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B52" t="str">
-        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
+        <v>polically exposed</v>
       </c>
       <c r="C52" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D52">
-        <v>1.16</v>
+        <v>2</v>
       </c>
       <c r="E52" t="str">
-        <v>cb4c27537d4c9ac33488c2d2d3ced67deb1ff4d8</v>
+        <v>50142c32072b7d8e388fd84c1502d1769de90711</v>
       </c>
       <c r="F52" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G52" t="str">
-        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
+        <v>polically exposed</v>
       </c>
       <c r="H52" t="str">
-        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
+        <v>polically exposed</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-10</v>
       </c>
       <c r="B53" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest liquid fund issue fix</v>
       </c>
       <c r="C53" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E53" t="str">
-        <v>N/A</v>
+        <v>ce45ff0a3a2bcea5d9f55790894c0dbf9ab9a78c</v>
       </c>
       <c r="F53" t="str">
-        <v>N/A</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G53" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest liquid fund issue fix</v>
       </c>
       <c r="H53" t="str">
-        <v>Daily Scrum Call</v>
+        <v>secureInvest liquid fund issue fix</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B54" t="str">
-        <v>DM-2394</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C54" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D54">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E54" t="str">
-        <v>a5ee1019cdcb541ec627f383ab6c9104045f048c</v>
+        <v>N/A</v>
       </c>
       <c r="F54" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G54" t="str">
-        <v>DM-2394</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H54" t="str">
-        <v>DM-2394</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B55" t="str">
-        <v>upload checkbox feature</v>
+        <v>uncheck dob feature</v>
       </c>
       <c r="C55" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D55">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E55" t="str">
-        <v>b502a004028755e9856792303ca1f5e33726b8a2</v>
+        <v>ead293f3b06815288e7967a7bb7e52107e7f6c94</v>
       </c>
       <c r="F55" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G55" t="str">
-        <v>upload checkbox feature</v>
+        <v>uncheck dob feature</v>
       </c>
       <c r="H55" t="str">
-        <v>upload checkbox feature</v>
+        <v>uncheck dob feature</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B56" t="str">
-        <v>Revert "address proof type also added"</v>
+        <v>adress flow change by enhancement</v>
       </c>
       <c r="C56" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D56">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E56" t="str">
-        <v>7ba1767399890d1c2cde14e5b2a6a743e86392ff</v>
+        <v>3097285a98b6d6a00da498f480f76072c6e1c592</v>
       </c>
       <c r="F56" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G56" t="str">
-        <v>Revert "address proof type also added"</v>
+        <v>adress flow change by enhancement</v>
       </c>
       <c r="H56" t="str">
-        <v>Revert "address proof type also added"</v>
+        <v>adress flow change by enhancement</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B57" t="str">
-        <v>address proof type also added</v>
+        <v>address enhanacement</v>
       </c>
       <c r="C57" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D57">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E57" t="str">
-        <v>62940a6c9d80db350938204b6164a4210a6329ca</v>
+        <v>1df15fe16d18561d9ae557d4af7f483a2d1939df</v>
       </c>
       <c r="F57" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G57" t="str">
-        <v>address proof type also added</v>
+        <v>address enhanacement</v>
       </c>
       <c r="H57" t="str">
-        <v>address proof type also added</v>
+        <v>address enhanacement</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B58" t="str">
-        <v>annur api fail navigateion</v>
+        <v>annur navigate to next even if api fail</v>
       </c>
       <c r="C58" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D58">
-        <v>1.33</v>
+        <v>1</v>
       </c>
       <c r="E58" t="str">
-        <v>ca7fe937e633709130fcf2b62edc7582dd30f9f6</v>
+        <v>c7f0f41075db3410129cceeaf5f971b6c742e667</v>
       </c>
       <c r="F58" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G58" t="str">
-        <v>annur api fail navigateion</v>
+        <v>annur navigate to next even if api fail</v>
       </c>
       <c r="H58" t="str">
-        <v>annur api fail navigateion</v>
+        <v>annur navigate to next even if api fail</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-06-15</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B59" t="str">
-        <v>add age proof as per DM-23374</v>
+        <v>add speical character validation on address</v>
       </c>
       <c r="C59" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D59">
-        <v>1.35</v>
+        <v>1</v>
       </c>
       <c r="E59" t="str">
-        <v>56f5281030fca42a747e2a596def58064e93f69e</v>
+        <v>a385b36d4af4fbaa692a2bb9c9b9d071bdf973d7</v>
       </c>
       <c r="F59" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G59" t="str">
-        <v>add age proof as per DM-23374</v>
+        <v>add speical character validation on address</v>
       </c>
       <c r="H59" t="str">
-        <v>add age proof as per DM-23374</v>
+        <v>add speical character validation on address</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-11</v>
       </c>
       <c r="B60" t="str">
-        <v>Daily Scrum Call</v>
+        <v>wealth edge issue fix</v>
       </c>
       <c r="C60" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E60" t="str">
-        <v>N/A</v>
+        <v>ac9e7046f9f21089761a6d96c097f94bb0ed7165</v>
       </c>
       <c r="F60" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G60" t="str">
-        <v>Daily Scrum Call</v>
+        <v>wealth edge issue fix</v>
       </c>
       <c r="H60" t="str">
-        <v>Daily Scrum Call</v>
+        <v>wealth edge issue fix</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B61" t="str">
-        <v>Dm-23443</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C61" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D61">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E61" t="str">
-        <v>f2fe5fcd220af0cf8bd4bc27899735ade613a321</v>
+        <v>N/A</v>
       </c>
       <c r="F61" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G61" t="str">
-        <v>Dm-23443</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H61" t="str">
-        <v>Dm-23443</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B62" t="str">
-        <v>DM-23381</v>
+        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
       </c>
       <c r="C62" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D62">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E62" t="str">
-        <v>ff9fd4f1691ccfc490c3d03f1c0095e68eefc42b</v>
+        <v>4f07e17fae2fa8cb32e3bf179b06b7e20fe8942f</v>
       </c>
       <c r="F62" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G62" t="str">
-        <v>DM-23381</v>
+        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
       </c>
       <c r="H62" t="str">
-        <v>DM-23381</v>
+        <v>If PO/LA is NRI but not mariner, current address outside India mandatory</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B63" t="str">
-        <v>pan validation error msg</v>
+        <v>pan number must be 10</v>
       </c>
       <c r="C63" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D63">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E63" t="str">
-        <v>d5a54a5cd7a0774aaf5d181e53979f5098e26522</v>
+        <v>6cf0060bb8f1341fd076662f36f21ea3ff1bf2e5</v>
       </c>
       <c r="F63" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G63" t="str">
-        <v>pan validation error msg</v>
+        <v>pan number must be 10</v>
       </c>
       <c r="H63" t="str">
-        <v>pan validation error msg</v>
+        <v>pan number must be 10</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B64" t="str">
-        <v>Non - School Going Child have value 185</v>
+        <v>Relationship with PEP other field add</v>
       </c>
       <c r="C64" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D64">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E64" t="str">
-        <v>25c68f96763134e98d0a9ea38a91c154157a7cfa</v>
+        <v>37de77bf0a1c9579237aa77cced98d5f64dfd18c</v>
       </c>
       <c r="F64" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G64" t="str">
-        <v>Non - School Going Child have value 185</v>
+        <v>Relationship with PEP other field add</v>
       </c>
       <c r="H64" t="str">
-        <v>Non - School Going Child have value 185</v>
+        <v>Relationship with PEP other field add</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B65" t="str">
-        <v>Dm-23443</v>
+        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
       </c>
       <c r="C65" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D65">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E65" t="str">
-        <v>3e07715dfd25da43ca278839e96c01e446ef161a</v>
+        <v>54688bbceecfe9edf3baff9717ace090b07f228f</v>
       </c>
       <c r="F65" t="str">
-        <v>infinityInsure2.0/uat</v>
+        <v>insure/develop</v>
       </c>
       <c r="G65" t="str">
-        <v>Dm-23443</v>
+        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
       </c>
       <c r="H65" t="str">
-        <v>Dm-23443</v>
+        <v>Employment questions for proposer should apply to LA; exclude if LA housewife</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-06-18</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B66" t="str">
-        <v>Daily Scrum Call</v>
+        <v>PO personal Health details should not come for form 2 cases</v>
       </c>
       <c r="C66" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D66">
         <v>1</v>
       </c>
       <c r="E66" t="str">
-        <v>N/A</v>
+        <v>d9b9549bf78158a844a9ce66cea71510c9ba251b</v>
       </c>
       <c r="F66" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G66" t="str">
-        <v>Daily Scrum Call</v>
+        <v>PO personal Health details should not come for form 2 cases</v>
       </c>
       <c r="H66" t="str">
-        <v>Daily Scrum Call</v>
+        <v>PO personal Health details should not come for form 2 cases</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-06-18</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B67" t="str">
-        <v>address checkbox fix</v>
+        <v>for 2 case questionior handle</v>
       </c>
       <c r="C67" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D67">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E67" t="str">
-        <v>407858e401bc2975e70bdf5856f6ab9b140f0960</v>
+        <v>09fd7f027227956b052b1b960c1097944cb1a60f</v>
       </c>
       <c r="F67" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G67" t="str">
-        <v>address checkbox fix</v>
+        <v>for 2 case questionior handle</v>
       </c>
       <c r="H67" t="str">
-        <v>address checkbox fix</v>
+        <v>for 2 case questionior handle</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-06-18</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B68" t="str">
-        <v>add address proof type</v>
+        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
       </c>
       <c r="C68" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D68">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E68" t="str">
-        <v>bdb0ea1853713cfe111eda9c06d8564bea6c2b79</v>
+        <v>cb4c27537d4c9ac33488c2d2d3ced67deb1ff4d8</v>
       </c>
       <c r="F68" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G68" t="str">
-        <v>add address proof type</v>
+        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
       </c>
       <c r="H68" t="str">
-        <v>add address proof type</v>
+        <v>If PO is Mariner, industry defaults to Merchant Marine (frozen)</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-06-19</v>
+        <v>2026-06-12</v>
       </c>
       <c r="B69" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Relationship with PEP other add</v>
       </c>
       <c r="C69" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D69">
         <v>1</v>
       </c>
       <c r="E69" t="str">
-        <v>N/A</v>
+        <v>4a4fd0af471fc6cda0950dba62dfb91d2f5d4660</v>
       </c>
       <c r="F69" t="str">
-        <v>N/A</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G69" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Relationship with PEP other add</v>
       </c>
       <c r="H69" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Relationship with PEP other add</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-06-19</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B70" t="str">
-        <v>tin number issue fix and proposal personal detail DM</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C70" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D70">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E70" t="str">
-        <v>a408a99385e9a653985a56f642fcc28ba2de57e0</v>
+        <v>N/A</v>
       </c>
       <c r="F70" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G70" t="str">
-        <v>tin number issue fix and proposal personal detail DM</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H70" t="str">
-        <v>tin number issue fix and proposal personal detail DM</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-06-22</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B71" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-2394</v>
       </c>
       <c r="C71" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D71">
         <v>1</v>
       </c>
       <c r="E71" t="str">
-        <v>N/A</v>
+        <v>a5ee1019cdcb541ec627f383ab6c9104045f048c</v>
       </c>
       <c r="F71" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G71" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-2394</v>
       </c>
       <c r="H71" t="str">
-        <v>Daily Scrum Call</v>
+        <v>DM-2394</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-06-22</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B72" t="str">
-        <v>single option auto select</v>
+        <v>upload checkbox feature</v>
       </c>
       <c r="C72" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" t="str">
-        <v>ec9dd5a17c8e072c718bc67e8f05ba8b58e90c53</v>
+        <v>b502a004028755e9856792303ca1f5e33726b8a2</v>
       </c>
       <c r="F72" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G72" t="str">
-        <v>single option auto select</v>
+        <v>upload checkbox feature</v>
       </c>
       <c r="H72" t="str">
-        <v>single option auto select</v>
+        <v>upload checkbox feature</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-06-22</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B73" t="str">
-        <v>dob check uncheck issue fix</v>
+        <v>Revert "address proof type also added"</v>
       </c>
       <c r="C73" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E73" t="str">
-        <v>d168932caf15589c1b9a12a597b27d05a0826231</v>
+        <v>7ba1767399890d1c2cde14e5b2a6a743e86392ff</v>
       </c>
       <c r="F73" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G73" t="str">
-        <v>dob check uncheck issue fix</v>
+        <v>Revert "address proof type also added"</v>
       </c>
       <c r="H73" t="str">
-        <v>dob check uncheck issue fix</v>
+        <v>Revert "address proof type also added"</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-06-22</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B74" t="str">
-        <v>age proof and address proof fix</v>
+        <v>address proof type also added</v>
       </c>
       <c r="C74" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74" t="str">
-        <v>08ac7ff4b44fa4830cd3fd240f46d549e398bf83</v>
+        <v>62940a6c9d80db350938204b6164a4210a6329ca</v>
       </c>
       <c r="F74" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G74" t="str">
-        <v>age proof and address proof fix</v>
+        <v>address proof type also added</v>
       </c>
       <c r="H74" t="str">
-        <v>age proof and address proof fix</v>
+        <v>address proof type also added</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-06-22</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B75" t="str">
-        <v>address type details</v>
+        <v>annur api fail navigateion</v>
       </c>
       <c r="C75" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E75" t="str">
-        <v>632f1d16ccc018a57846aed8211535da54451d74</v>
+        <v>ca7fe937e633709130fcf2b62edc7582dd30f9f6</v>
       </c>
       <c r="F75" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G75" t="str">
-        <v>address type details</v>
+        <v>annur api fail navigateion</v>
       </c>
       <c r="H75" t="str">
-        <v>address type details</v>
+        <v>annur api fail navigateion</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B76" t="str">
-        <v>Daily Scrum Call</v>
+        <v>add age proof as per DM-23374</v>
       </c>
       <c r="C76" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D76">
         <v>1</v>
       </c>
       <c r="E76" t="str">
-        <v>N/A</v>
+        <v>56f5281030fca42a747e2a596def58064e93f69e</v>
       </c>
       <c r="F76" t="str">
-        <v>N/A</v>
+        <v>insure/develop</v>
       </c>
       <c r="G76" t="str">
-        <v>Daily Scrum Call</v>
+        <v>add age proof as per DM-23374</v>
       </c>
       <c r="H76" t="str">
-        <v>Daily Scrum Call</v>
+        <v>add age proof as per DM-23374</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B77" t="str">
-        <v>heading driver question</v>
+        <v>Revert "address proff type also added"</v>
       </c>
       <c r="C77" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D77">
-        <v>2.67</v>
+        <v>1</v>
       </c>
       <c r="E77" t="str">
-        <v>6fb9c4b7629345c302e7ec197ca778d0ef9846cc</v>
+        <v>ff7e09dae9e6ac17225ec0da9a3734621b2ec3b9</v>
       </c>
       <c r="F77" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G77" t="str">
-        <v>heading driver question</v>
+        <v>Revert "address proff type also added"</v>
       </c>
       <c r="H77" t="str">
-        <v>heading driver question</v>
+        <v>Revert "address proff type also added"</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B78" t="str">
-        <v>driver questionar</v>
+        <v>Revert "address proff type also added"</v>
       </c>
       <c r="C78" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D78">
-        <v>2.67</v>
+        <v>1</v>
       </c>
       <c r="E78" t="str">
-        <v>2d63fc872425b4c874f97a3dfb2dbafe543b892d</v>
+        <v>719d86992602a3df2a1f779bfd31c67b6e62ef45</v>
       </c>
       <c r="F78" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G78" t="str">
-        <v>driver questionar</v>
+        <v>Revert "address proff type also added"</v>
       </c>
       <c r="H78" t="str">
-        <v>driver questionar</v>
+        <v>Revert "address proff type also added"</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-15</v>
       </c>
       <c r="B79" t="str">
-        <v>DM-23546</v>
+        <v>address proff type also added</v>
       </c>
       <c r="C79" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D79">
-        <v>2.66</v>
+        <v>0</v>
       </c>
       <c r="E79" t="str">
-        <v>e2fca5aca7bbd4758ad5ff5bb7331aa403f5c405</v>
+        <v>85c5e918bb5e2b78022008315fd0d5fe21b6d545</v>
       </c>
       <c r="F79" t="str">
-        <v>insure/develop</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G79" t="str">
-        <v>DM-23546</v>
+        <v>address proff type also added</v>
       </c>
       <c r="H79" t="str">
-        <v>DM-23546</v>
+        <v>address proff type also added</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B80" t="str">
         <v>Daily Scrum Call</v>
@@ -2481,371 +2482,1203 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B81" t="str">
-        <v>address and dob always unchecked</v>
+        <v>Dm-23443</v>
       </c>
       <c r="C81" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E81" t="str">
-        <v>b4a7f1a6f3ef2cc5efbcc6f5b78dea8804a24a24</v>
+        <v>f2fe5fcd220af0cf8bd4bc27899735ade613a321</v>
       </c>
       <c r="F81" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G81" t="str">
-        <v>address and dob always unchecked</v>
+        <v>Dm-23443</v>
       </c>
       <c r="H81" t="str">
-        <v>address and dob always unchecked</v>
+        <v>Dm-23443</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B82" t="str">
-        <v>promise4growthplus DM fixes</v>
+        <v>DM-23381</v>
       </c>
       <c r="C82" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D82">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E82" t="str">
-        <v>b7b3a18ef18378d3c993910abd73ed738440ad3e</v>
+        <v>ff9fd4f1691ccfc490c3d03f1c0095e68eefc42b</v>
       </c>
       <c r="F82" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G82" t="str">
-        <v>promise4growthplus DM fixes</v>
+        <v>DM-23381</v>
       </c>
       <c r="H82" t="str">
-        <v>promise4growthplus DM fixes</v>
+        <v>DM-23381</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B83" t="str">
-        <v>dock question multiselect</v>
+        <v>pan validation error msg</v>
       </c>
       <c r="C83" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E83" t="str">
-        <v>c28f1368399b3c0d8e8f0a3bd21a660001c1ac3f</v>
+        <v>d5a54a5cd7a0774aaf5d181e53979f5098e26522</v>
       </c>
       <c r="F83" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G83" t="str">
-        <v>dock question multiselect</v>
+        <v>pan validation error msg</v>
       </c>
       <c r="H83" t="str">
-        <v>dock question multiselect</v>
+        <v>pan validation error msg</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B84" t="str">
-        <v>LA Medical Details come for form 2 case only</v>
+        <v>Non - School Going Child have value 185</v>
       </c>
       <c r="C84" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D84">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E84" t="str">
-        <v>6d9049c8e776a726ab2e2cadf8d2f77ccf2c803d</v>
+        <v>25c68f96763134e98d0a9ea38a91c154157a7cfa</v>
       </c>
       <c r="F84" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G84" t="str">
-        <v>LA Medical Details come for form 2 case only</v>
+        <v>Non - School Going Child have value 185</v>
       </c>
       <c r="H84" t="str">
-        <v>LA Medical Details come for form 2 case only</v>
+        <v>Non - School Going Child have value 185</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-06-26</v>
+        <v>2026-06-16</v>
       </c>
       <c r="B85" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Dm-23443</v>
       </c>
       <c r="C85" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E85" t="str">
-        <v>N/A</v>
+        <v>3e07715dfd25da43ca278839e96c01e446ef161a</v>
       </c>
       <c r="F85" t="str">
-        <v>N/A</v>
+        <v>infinityInsure2.0/uat</v>
       </c>
       <c r="G85" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Dm-23443</v>
       </c>
       <c r="H85" t="str">
-        <v>Daily Scrum Call</v>
+        <v>Dm-23443</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-06-26</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B86" t="str">
-        <v>ulip rider plan code</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C86" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D86">
-        <v>2.67</v>
+        <v>1</v>
       </c>
       <c r="E86" t="str">
-        <v>84f93450837775e7e63ee19b1ab48edbb7039310</v>
+        <v>N/A</v>
       </c>
       <c r="F86" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G86" t="str">
-        <v>ulip rider plan code</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H86" t="str">
-        <v>ulip rider plan code</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-06-26</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B87" t="str">
-        <v>dont show harcoded error message on annur</v>
+        <v>address checkbox fix</v>
       </c>
       <c r="C87" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D87">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="E87" t="str">
-        <v>e22e159cd06c15111919b9408eb0d1435b301574</v>
+        <v>407858e401bc2975e70bdf5856f6ab9b140f0960</v>
       </c>
       <c r="F87" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G87" t="str">
-        <v>dont show harcoded error message on annur</v>
+        <v>address checkbox fix</v>
       </c>
       <c r="H87" t="str">
-        <v>dont show harcoded error message on annur</v>
+        <v>address checkbox fix</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-06-26</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B88" t="str">
-        <v>when no rider directly continue</v>
+        <v>add address proof type</v>
       </c>
       <c r="C88" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D88">
-        <v>2.66</v>
+        <v>2</v>
       </c>
       <c r="E88" t="str">
-        <v>c250ba72d7414c93b52250f1a5bbc227aae3d2a0</v>
+        <v>bdb0ea1853713cfe111eda9c06d8564bea6c2b79</v>
       </c>
       <c r="F88" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G88" t="str">
-        <v>when no rider directly continue</v>
+        <v>add address proof type</v>
       </c>
       <c r="H88" t="str">
-        <v>when no rider directly continue</v>
+        <v>add address proof type</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-06-29</v>
+        <v>2026-06-18</v>
       </c>
       <c r="B89" t="str">
-        <v>Daily Scrum Call</v>
+        <v>address type mapping</v>
       </c>
       <c r="C89" t="str">
-        <v>Meeting</v>
+        <v>Development &amp; Configuration</v>
       </c>
       <c r="D89">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E89" t="str">
-        <v>N/A</v>
+        <v>b405ff6497eaf2fb030c2fed60e43d391b9a8e80</v>
       </c>
       <c r="F89" t="str">
-        <v>N/A</v>
+        <v>uat-common-backend-1</v>
       </c>
       <c r="G89" t="str">
-        <v>Daily Scrum Call</v>
+        <v>address type mapping</v>
       </c>
       <c r="H89" t="str">
-        <v>Daily Scrum Call</v>
+        <v>address type mapping</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-06-29</v>
+        <v>2026-06-19</v>
       </c>
       <c r="B90" t="str">
-        <v>open numeric keypad in suatabilyt matrix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C90" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D90">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E90" t="str">
-        <v>f64f202e90af5d1099e59d83d57f070f934b0d13</v>
+        <v>N/A</v>
       </c>
       <c r="F90" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G90" t="str">
-        <v>open numeric keypad in suatabilyt matrix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H90" t="str">
-        <v>open numeric keypad in suatabilyt matrix</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-06-29</v>
+        <v>2026-06-19</v>
       </c>
       <c r="B91" t="str">
-        <v>error on generate BI also condiser gernal error</v>
+        <v>tin number issue fix and proposal personal detail DM</v>
       </c>
       <c r="C91" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D91">
-        <v>1.6</v>
+        <v>8</v>
       </c>
       <c r="E91" t="str">
-        <v>48b28334b39accca8f60e61d842d2e08b2e88210</v>
+        <v>a408a99385e9a653985a56f642fcc28ba2de57e0</v>
       </c>
       <c r="F91" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G91" t="str">
-        <v>error on generate BI also condiser gernal error</v>
+        <v>tin number issue fix and proposal personal detail DM</v>
       </c>
       <c r="H91" t="str">
-        <v>error on generate BI also condiser gernal error</v>
+        <v>tin number issue fix and proposal personal detail DM</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-06-29</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B92" t="str">
-        <v>promise4growthplus ppt value isssue fix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="C92" t="str">
-        <v>Development &amp; Configuration</v>
+        <v>Meeting</v>
       </c>
       <c r="D92">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E92" t="str">
-        <v>8d7da8462d1558b346eafda60080e9e917abdc18</v>
+        <v>N/A</v>
       </c>
       <c r="F92" t="str">
-        <v>insure/develop</v>
+        <v>N/A</v>
       </c>
       <c r="G92" t="str">
-        <v>promise4growthplus ppt value isssue fix</v>
+        <v>Daily Scrum Call</v>
       </c>
       <c r="H92" t="str">
-        <v>promise4growthplus ppt value isssue fix</v>
+        <v>Daily Scrum Call</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-06-29</v>
+        <v>2026-06-22</v>
       </c>
       <c r="B93" t="str">
-        <v>height,weight decial logic same as ISNP</v>
+        <v>single option auto select</v>
       </c>
       <c r="C93" t="str">
         <v>Development &amp; Configuration</v>
       </c>
       <c r="D93">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E93" t="str">
-        <v>4dfa9dd3d803e4ec3ea56f32a63850c2a4bcbbd7</v>
+        <v>ec9dd5a17c8e072c718bc67e8f05ba8b58e90c53</v>
       </c>
       <c r="F93" t="str">
         <v>insure/develop</v>
       </c>
       <c r="G93" t="str">
-        <v>height,weight decial logic same as ISNP</v>
+        <v>single option auto select</v>
       </c>
       <c r="H93" t="str">
-        <v>height,weight decial logic same as ISNP</v>
+        <v>single option auto select</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="B94" t="str">
+        <v>dob check uncheck issue fix</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94" t="str">
+        <v>d168932caf15589c1b9a12a597b27d05a0826231</v>
+      </c>
+      <c r="F94" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G94" t="str">
+        <v>dob check uncheck issue fix</v>
+      </c>
+      <c r="H94" t="str">
+        <v>dob check uncheck issue fix</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="B95" t="str">
+        <v>age proof and address proof fix</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95" t="str">
+        <v>08ac7ff4b44fa4830cd3fd240f46d549e398bf83</v>
+      </c>
+      <c r="F95" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G95" t="str">
+        <v>age proof and address proof fix</v>
+      </c>
+      <c r="H95" t="str">
+        <v>age proof and address proof fix</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="B96" t="str">
+        <v>address type details</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D96">
+        <v>1</v>
+      </c>
+      <c r="E96" t="str">
+        <v>632f1d16ccc018a57846aed8211535da54451d74</v>
+      </c>
+      <c r="F96" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G96" t="str">
+        <v>address type details</v>
+      </c>
+      <c r="H96" t="str">
+        <v>address type details</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="B97" t="str">
+        <v>age proof and address proof fix</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+      <c r="E97" t="str">
+        <v>b11d955f30d2894156ee9eb98245716aee19704f</v>
+      </c>
+      <c r="F97" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G97" t="str">
+        <v>age proof and address proof fix</v>
+      </c>
+      <c r="H97" t="str">
+        <v>age proof and address proof fix</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="B98" t="str">
+        <v>address type details</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D98">
+        <v>3</v>
+      </c>
+      <c r="E98" t="str">
+        <v>3a837721569e94449274103a7ec882e69bc4e14d</v>
+      </c>
+      <c r="F98" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G98" t="str">
+        <v>address type details</v>
+      </c>
+      <c r="H98" t="str">
+        <v>address type details</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F99" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G99" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="H99" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="B100" t="str">
+        <v>heading driver question</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D100">
+        <v>2</v>
+      </c>
+      <c r="E100" t="str">
+        <v>6fb9c4b7629345c302e7ec197ca778d0ef9846cc</v>
+      </c>
+      <c r="F100" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G100" t="str">
+        <v>heading driver question</v>
+      </c>
+      <c r="H100" t="str">
+        <v>heading driver question</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="B101" t="str">
+        <v>driver questionar</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D101">
+        <v>2</v>
+      </c>
+      <c r="E101" t="str">
+        <v>2d63fc872425b4c874f97a3dfb2dbafe543b892d</v>
+      </c>
+      <c r="F101" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G101" t="str">
+        <v>driver questionar</v>
+      </c>
+      <c r="H101" t="str">
+        <v>driver questionar</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="B102" t="str">
+        <v>DM-23546</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D102">
+        <v>2</v>
+      </c>
+      <c r="E102" t="str">
+        <v>e2fca5aca7bbd4758ad5ff5bb7331aa403f5c405</v>
+      </c>
+      <c r="F102" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G102" t="str">
+        <v>DM-23546</v>
+      </c>
+      <c r="H102" t="str">
+        <v>DM-23546</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="B103" t="str">
+        <v>driver questioner</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D103">
+        <v>2</v>
+      </c>
+      <c r="E103" t="str">
+        <v>6cf47321a603e9d5f4e71d9b3b245c3744a9e8b9</v>
+      </c>
+      <c r="F103" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G103" t="str">
+        <v>driver questioner</v>
+      </c>
+      <c r="H103" t="str">
+        <v>driver questioner</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
+      </c>
+      <c r="E104" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F104" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="H104" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B105" t="str">
+        <v>address and dob always unchecked</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D105">
+        <v>2</v>
+      </c>
+      <c r="E105" t="str">
+        <v>b4a7f1a6f3ef2cc5efbcc6f5b78dea8804a24a24</v>
+      </c>
+      <c r="F105" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G105" t="str">
+        <v>address and dob always unchecked</v>
+      </c>
+      <c r="H105" t="str">
+        <v>address and dob always unchecked</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B106" t="str">
+        <v>promise4growthplus DM fixes</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D106">
+        <v>2</v>
+      </c>
+      <c r="E106" t="str">
+        <v>b7b3a18ef18378d3c993910abd73ed738440ad3e</v>
+      </c>
+      <c r="F106" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G106" t="str">
+        <v>promise4growthplus DM fixes</v>
+      </c>
+      <c r="H106" t="str">
+        <v>promise4growthplus DM fixes</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B107" t="str">
+        <v>dock question multiselect</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D107">
+        <v>2</v>
+      </c>
+      <c r="E107" t="str">
+        <v>c28f1368399b3c0d8e8f0a3bd21a660001c1ac3f</v>
+      </c>
+      <c r="F107" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G107" t="str">
+        <v>dock question multiselect</v>
+      </c>
+      <c r="H107" t="str">
+        <v>dock question multiselect</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="B108" t="str">
+        <v>LA Medical Details come for form 2 case only</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D108">
+        <v>2</v>
+      </c>
+      <c r="E108" t="str">
+        <v>6d9049c8e776a726ab2e2cadf8d2f77ccf2c803d</v>
+      </c>
+      <c r="F108" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G108" t="str">
+        <v>LA Medical Details come for form 2 case only</v>
+      </c>
+      <c r="H108" t="str">
+        <v>LA Medical Details come for form 2 case only</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D109">
+        <v>1</v>
+      </c>
+      <c r="E109" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F109" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G109" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="H109" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B110" t="str">
+        <v>ulip rider plan code</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D110">
+        <v>1</v>
+      </c>
+      <c r="E110" t="str">
+        <v>84f93450837775e7e63ee19b1ab48edbb7039310</v>
+      </c>
+      <c r="F110" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G110" t="str">
+        <v>ulip rider plan code</v>
+      </c>
+      <c r="H110" t="str">
+        <v>ulip rider plan code</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B111" t="str">
+        <v>dont show harcoded error message on annur</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D111">
+        <v>1</v>
+      </c>
+      <c r="E111" t="str">
+        <v>e22e159cd06c15111919b9408eb0d1435b301574</v>
+      </c>
+      <c r="F111" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G111" t="str">
+        <v>dont show harcoded error message on annur</v>
+      </c>
+      <c r="H111" t="str">
+        <v>dont show harcoded error message on annur</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B112" t="str">
+        <v>when no rider directly continue</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D112">
+        <v>1</v>
+      </c>
+      <c r="E112" t="str">
+        <v>c250ba72d7414c93b52250f1a5bbc227aae3d2a0</v>
+      </c>
+      <c r="F112" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G112" t="str">
+        <v>when no rider directly continue</v>
+      </c>
+      <c r="H112" t="str">
+        <v>when no rider directly continue</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B113" t="str">
+        <v>rider plan code for ulip</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D113">
+        <v>1</v>
+      </c>
+      <c r="E113" t="str">
+        <v>50643aac33cb3566db6c57c19a81eec756aa7af0</v>
+      </c>
+      <c r="F113" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G113" t="str">
+        <v>rider plan code for ulip</v>
+      </c>
+      <c r="H113" t="str">
+        <v>rider plan code for ulip</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="B114" t="str">
+        <v>SPF PDF Product name is Missing</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D114">
+        <v>4</v>
+      </c>
+      <c r="E114" t="str">
+        <v>afd2e3d7ee62e112e81ff865b9269a8ab1bbf3d4</v>
+      </c>
+      <c r="F114" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G114" t="str">
+        <v>SPF PDF Product name is Missing</v>
+      </c>
+      <c r="H114" t="str">
+        <v>SPF PDF Product name is Missing</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
         <v>2026-06-29</v>
       </c>
-      <c r="B94" t="str">
+      <c r="B115" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D115">
+        <v>1</v>
+      </c>
+      <c r="E115" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F115" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="H115" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B116" t="str">
+        <v>open numeric keypad in suatabilyt matrix</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D116">
+        <v>1</v>
+      </c>
+      <c r="E116" t="str">
+        <v>f64f202e90af5d1099e59d83d57f070f934b0d13</v>
+      </c>
+      <c r="F116" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G116" t="str">
+        <v>open numeric keypad in suatabilyt matrix</v>
+      </c>
+      <c r="H116" t="str">
+        <v>open numeric keypad in suatabilyt matrix</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B117" t="str">
+        <v>error on generate BI also condiser gernal error</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D117">
+        <v>1</v>
+      </c>
+      <c r="E117" t="str">
+        <v>48b28334b39accca8f60e61d842d2e08b2e88210</v>
+      </c>
+      <c r="F117" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G117" t="str">
+        <v>error on generate BI also condiser gernal error</v>
+      </c>
+      <c r="H117" t="str">
+        <v>error on generate BI also condiser gernal error</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B118" t="str">
+        <v>promise4growthplus ppt value isssue fix</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D118">
+        <v>1</v>
+      </c>
+      <c r="E118" t="str">
+        <v>8d7da8462d1558b346eafda60080e9e917abdc18</v>
+      </c>
+      <c r="F118" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G118" t="str">
+        <v>promise4growthplus ppt value isssue fix</v>
+      </c>
+      <c r="H118" t="str">
+        <v>promise4growthplus ppt value isssue fix</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B119" t="str">
+        <v>height,weight decial logic same as ISNP</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D119">
+        <v>1</v>
+      </c>
+      <c r="E119" t="str">
+        <v>4dfa9dd3d803e4ec3ea56f32a63850c2a4bcbbd7</v>
+      </c>
+      <c r="F119" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G119" t="str">
+        <v>height,weight decial logic same as ISNP</v>
+      </c>
+      <c r="H119" t="str">
+        <v>height,weight decial logic same as ISNP</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="B120" t="str">
         <v>training api byass temp</v>
       </c>
-      <c r="C94" t="str">
-        <v>Development &amp; Configuration</v>
-      </c>
-      <c r="D94">
-        <v>1.6</v>
-      </c>
-      <c r="E94" t="str">
+      <c r="C120" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D120">
+        <v>4</v>
+      </c>
+      <c r="E120" t="str">
         <v>9a8e40da79daed6e65fd0e6ae77f596a4852e663</v>
       </c>
-      <c r="F94" t="str">
-        <v>insure/develop</v>
-      </c>
-      <c r="G94" t="str">
+      <c r="F120" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G120" t="str">
         <v>training api byass temp</v>
       </c>
-      <c r="H94" t="str">
+      <c r="H120" t="str">
         <v>training api byass temp</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D121">
+        <v>1</v>
+      </c>
+      <c r="E121" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F121" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G121" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="H121" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B122" t="str">
+        <v>tpa api integration</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D122">
+        <v>2</v>
+      </c>
+      <c r="E122" t="str">
+        <v>4fdf6e55e458c3a76f5390445d65db36ff5fda3e</v>
+      </c>
+      <c r="F122" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G122" t="str">
+        <v>tpa api integration</v>
+      </c>
+      <c r="H122" t="str">
+        <v>tpa api integration</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B123" t="str">
+        <v>tpa api  integration</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D123">
+        <v>2</v>
+      </c>
+      <c r="E123" t="str">
+        <v>74d1761fc719b203749a19a33d9d9b9707b0fbd1</v>
+      </c>
+      <c r="F123" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G123" t="str">
+        <v>tpa api  integration</v>
+      </c>
+      <c r="H123" t="str">
+        <v>tpa api  integration</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="B124" t="str">
+        <v>DM-23544</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D124">
+        <v>4</v>
+      </c>
+      <c r="E124" t="str">
+        <v>9420abfa690ba5fa1db8814f3c68083639216de2</v>
+      </c>
+      <c r="F124" t="str">
+        <v>insure/develop</v>
+      </c>
+      <c r="G124" t="str">
+        <v>DM-23544</v>
+      </c>
+      <c r="H124" t="str">
+        <v>DM-23544</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="D125">
+        <v>1</v>
+      </c>
+      <c r="E125" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F125" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G125" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+      <c r="H125" t="str">
+        <v>Daily Scrum Call</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="B126" t="str">
+        <v>fix(insure): enhance staff discount normalization logic</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Development &amp; Configuration</v>
+      </c>
+      <c r="D126">
+        <v>8</v>
+      </c>
+      <c r="E126" t="str">
+        <v>3c6612d1fe2fd0fcef05bdb56c7836af5b9d6ccf</v>
+      </c>
+      <c r="F126" t="str">
+        <v>uat-common-backend-1</v>
+      </c>
+      <c r="G126" t="str">
+        <v>fix(insure): enhance staff discount normalization logic</v>
+      </c>
+      <c r="H126" t="str">
+        <v>fix(insure): enhance staff discount normalization logic</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H126"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>